<commit_message>
fix: use relative paths in experiment tracker hyperlinks and cells
</commit_message>
<xml_diff>
--- a/experiment_tracker.xlsx
+++ b/experiment_tracker.xlsx
@@ -1544,7 +1544,7 @@
         <v>-0.06560000000000001</v>
       </c>
       <c r="D2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -1568,7 +1568,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE2"/>
+  <dimension ref="A1:AE3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1888,6 +1888,133 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-04-10 18:46</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>GB1_additive</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>python scripts/run_integrated_gradients.py configs/synthetic/GB1_additive_config.yaml</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>configs/synthetic/GB1_additive_config.yaml</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_additive_LINEAR/GB1_additive_config_snapshot_20260410_181528.yaml</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_additive_LINEAR</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_additive_LINEAR/GB1_additive_run_log_20260410_181528.txt</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>esm_attention</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>256-128-64-32</t>
+        </is>
+      </c>
+      <c r="K3" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="M3" t="n">
+        <v>64</v>
+      </c>
+      <c r="N3" t="n">
+        <v>50</v>
+      </c>
+      <c r="O3" t="n">
+        <v>10</v>
+      </c>
+      <c r="P3" t="n">
+        <v>15</v>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>huber</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="S3" s="2" t="n">
+        <v>-0.0003</v>
+      </c>
+      <c r="T3" t="n">
+        <v>0.0061</v>
+      </c>
+      <c r="U3" s="2" t="n">
+        <v>0.0232</v>
+      </c>
+      <c r="V3" t="n">
+        <v>0.0402</v>
+      </c>
+      <c r="W3" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="X3" s="2" t="n">
+        <v>-0.0425</v>
+      </c>
+      <c r="Y3" s="2" t="n">
+        <v>-0.1654</v>
+      </c>
+      <c r="Z3" s="2" t="n">
+        <v>-0.06560000000000001</v>
+      </c>
+      <c r="AA3" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_additive_LINEAR/GB1_additive_cv_loss_curves.png</t>
+        </is>
+      </c>
+      <c r="AB3" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_additive_LINEAR/GB1_additive_predicted_vs_actual_test.png</t>
+        </is>
+      </c>
+      <c r="AC3" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_additive_LINEAR/GB1_additive_integrated_gradients_heatmap.png</t>
+        </is>
+      </c>
+      <c r="AD3" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_additive_LINEAR/GB1_additive_integrated_gradients_analysis.png</t>
+        </is>
+      </c>
+      <c r="AE3" t="inlineStr">
+        <is>
+          <t>new MLP architecture</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F2" r:id="rId1"/>
@@ -1896,6 +2023,12 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB2" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC2" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD2" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F3" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H3" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA3" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB3" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC3" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD3" r:id="rId12"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Added first row of p53 epistatic and nonlinear
</commit_message>
<xml_diff>
--- a/experiment_tracker.xlsx
+++ b/experiment_tracker.xlsx
@@ -1754,7 +1754,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1862,16 +1862,68 @@
         <v>0.2194</v>
       </c>
       <c r="D4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>2026-04-12 09:15</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>results/synthetic/p53_additive_LINEAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>p53_epistatic</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="n">
+        <v>0.7277</v>
+      </c>
+      <c r="C5" s="5" t="n">
+        <v>0.2497</v>
+      </c>
+      <c r="D5" t="n">
         <v>1</v>
       </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>2026-04-12 09:15</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>results/synthetic/p53_additive_LINEAR</t>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>2026-04-12 17:34</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>results/synthetic/p53_epistatic_LINEAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>p53_nonlinear</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="n">
+        <v>0.7762</v>
+      </c>
+      <c r="C6" s="5" t="n">
+        <v>0.2073</v>
+      </c>
+      <c r="D6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>2026-04-12 17:34</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>results/synthetic/p53_nonlinear_LINEAR</t>
         </is>
       </c>
     </row>
@@ -2766,6 +2818,478 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:AE3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="7" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="45" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="45" customWidth="1" min="7" max="7"/>
+    <col width="45" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="8" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
+    <col width="10" customWidth="1" min="16" max="16"/>
+    <col width="12" customWidth="1" min="17" max="17"/>
+    <col width="14" customWidth="1" min="18" max="18"/>
+    <col width="16" customWidth="1" min="19" max="19"/>
+    <col width="14" customWidth="1" min="20" max="20"/>
+    <col width="20" customWidth="1" min="21" max="21"/>
+    <col width="18" customWidth="1" min="22" max="22"/>
+    <col width="18" customWidth="1" min="23" max="23"/>
+    <col width="10" customWidth="1" min="24" max="24"/>
+    <col width="15" customWidth="1" min="25" max="25"/>
+    <col width="16" customWidth="1" min="26" max="26"/>
+    <col width="20" customWidth="1" min="27" max="27"/>
+    <col width="22" customWidth="1" min="28" max="28"/>
+    <col width="18" customWidth="1" min="29" max="29"/>
+    <col width="18" customWidth="1" min="30" max="30"/>
+    <col width="40" customWidth="1" min="31" max="31"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Run #</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Timestamp</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Dataset</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Command</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Config (input)</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Config snapshot</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Results dir</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Run log</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>pooling_method</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>hidden_dims</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>dropout_rate</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>learning_rate</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>batch_size</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>epochs</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>min_epochs</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>patience</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>loss_type</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>normalization</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>CV mean val R²</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>CV std val R²</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>CV mean val Spearman</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>CV std val Spearman</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>CV avg best epoch</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>Test R²</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>Test Pearson r</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>Test Spearman ρ</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>CV loss curves</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>Test pred vs actual</t>
+        </is>
+      </c>
+      <c r="AC1" s="1" t="inlineStr">
+        <is>
+          <t>IG heatmap</t>
+        </is>
+      </c>
+      <c r="AD1" s="1" t="inlineStr">
+        <is>
+          <t>IG analysis</t>
+        </is>
+      </c>
+      <c r="AE1" s="1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2026-04-12 09:15</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>p53_additive</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>python scripts/run_integrated_gradients.py configs/synthetic/p53_additive_config.yaml</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>configs/synthetic/p53_additive_config.yaml</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/p53_additive_LINEAR/p53_additive_config_snapshot_20260412_012304.yaml</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>results/synthetic/p53_additive_LINEAR</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/p53_additive_LINEAR/p53_additive_run_log_20260412_012304.txt</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>esm_attention</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>1024-512-256-128</t>
+        </is>
+      </c>
+      <c r="K2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0.0005</v>
+      </c>
+      <c r="M2" t="n">
+        <v>256</v>
+      </c>
+      <c r="N2" t="n">
+        <v>50</v>
+      </c>
+      <c r="O2" t="n">
+        <v>10</v>
+      </c>
+      <c r="P2" t="n">
+        <v>15</v>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>huber</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="S2" s="4" t="n">
+        <v>0.6383</v>
+      </c>
+      <c r="T2" t="n">
+        <v>0.0736</v>
+      </c>
+      <c r="U2" s="5" t="n">
+        <v>0.2053</v>
+      </c>
+      <c r="V2" t="n">
+        <v>0.0231</v>
+      </c>
+      <c r="W2" t="n">
+        <v>47.6</v>
+      </c>
+      <c r="X2" s="4" t="n">
+        <v>0.7309</v>
+      </c>
+      <c r="Y2" s="4" t="n">
+        <v>0.8561</v>
+      </c>
+      <c r="Z2" s="5" t="n">
+        <v>0.2194</v>
+      </c>
+      <c r="AA2" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/p53_additive_LINEAR/p53_additive_cv_loss_curves.png</t>
+        </is>
+      </c>
+      <c r="AB2" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/p53_additive_LINEAR/p53_additive_predicted_vs_actual_test.png</t>
+        </is>
+      </c>
+      <c r="AC2" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/p53_additive_LINEAR/p53_additive_integrated_gradients_heatmap.png</t>
+        </is>
+      </c>
+      <c r="AD2" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/p53_additive_LINEAR/p53_additive_integrated_gradients_analysis.png</t>
+        </is>
+      </c>
+      <c r="AE2" t="inlineStr">
+        <is>
+          <t>First p53 after OOOM</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-04-12 17:28</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>p53_additive</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>python scripts/run_integrated_gradients.py configs/synthetic/p53_additive_config.yaml</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>configs/synthetic/p53_additive_config.yaml</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/p53_additive_LINEAR/p53_additive_config_snapshot_20260412_140326.yaml</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>results/synthetic/p53_additive_LINEAR</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/p53_additive_LINEAR/p53_additive_run_log_20260412_140326.txt</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>esm_attention</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>2056-1024-512-256</t>
+        </is>
+      </c>
+      <c r="K3" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0.0005</v>
+      </c>
+      <c r="M3" t="n">
+        <v>256</v>
+      </c>
+      <c r="N3" t="n">
+        <v>50</v>
+      </c>
+      <c r="O3" t="n">
+        <v>15</v>
+      </c>
+      <c r="P3" t="n">
+        <v>30</v>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>huber</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="S3" s="4" t="n">
+        <v>0.5503</v>
+      </c>
+      <c r="T3" t="n">
+        <v>0.1706</v>
+      </c>
+      <c r="U3" s="5" t="n">
+        <v>0.2316</v>
+      </c>
+      <c r="V3" t="n">
+        <v>0.0728</v>
+      </c>
+      <c r="W3" t="n">
+        <v>46.6</v>
+      </c>
+      <c r="X3" s="4" t="n">
+        <v>0.6378</v>
+      </c>
+      <c r="Y3" s="4" t="n">
+        <v>0.8038</v>
+      </c>
+      <c r="Z3" s="2" t="n">
+        <v>0.1813</v>
+      </c>
+      <c r="AA3" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/p53_additive_LINEAR/p53_additive_cv_loss_curves.png</t>
+        </is>
+      </c>
+      <c r="AB3" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/p53_additive_LINEAR/p53_additive_predicted_vs_actual_test.png</t>
+        </is>
+      </c>
+      <c r="AC3" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/p53_additive_LINEAR/p53_additive_integrated_gradients_heatmap.png</t>
+        </is>
+      </c>
+      <c r="AD3" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/p53_additive_LINEAR/p53_additive_integrated_gradients_analysis.png</t>
+        </is>
+      </c>
+      <c r="AE3" t="inlineStr">
+        <is>
+          <t>p53 additive 2</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H2" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA2" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB2" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC2" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD2" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F3" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H3" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA3" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB3" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC3" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD3" r:id="rId12"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:AE2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -2965,37 +3489,37 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-04-12 09:15</t>
+          <t>2026-04-12 17:34</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>p53_additive</t>
+          <t>p53_epistatic</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>python scripts/run_integrated_gradients.py configs/synthetic/p53_additive_config.yaml</t>
+          <t>python scripts/run_integrated_gradients.py configs/synthetic/p53_epistatic_config.yaml</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>configs/synthetic/p53_additive_config.yaml</t>
+          <t>configs/synthetic/p53_epistatic_config.yaml</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>results/synthetic/p53_additive_LINEAR/p53_additive_config_snapshot_20260412_012304.yaml</t>
+          <t>results/synthetic/p53_epistatic_LINEAR/p53_epistatic_config_snapshot_20260412_095552.yaml</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>results/synthetic/p53_additive_LINEAR</t>
+          <t>results/synthetic/p53_epistatic_LINEAR</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>results/synthetic/p53_additive_LINEAR/p53_additive_run_log_20260412_012304.txt</t>
+          <t>results/synthetic/p53_epistatic_LINEAR/p53_epistatic_run_log_20260412_095552.txt</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -3037,52 +3561,52 @@
         </is>
       </c>
       <c r="S2" s="4" t="n">
-        <v>0.6383</v>
+        <v>0.5198</v>
       </c>
       <c r="T2" t="n">
-        <v>0.0736</v>
+        <v>0.1104</v>
       </c>
       <c r="U2" s="5" t="n">
-        <v>0.2053</v>
+        <v>0.2172</v>
       </c>
       <c r="V2" t="n">
-        <v>0.0231</v>
+        <v>0.0433</v>
       </c>
       <c r="W2" t="n">
-        <v>47.6</v>
+        <v>45.2</v>
       </c>
       <c r="X2" s="4" t="n">
-        <v>0.7309</v>
+        <v>0.7277</v>
       </c>
       <c r="Y2" s="4" t="n">
-        <v>0.8561</v>
+        <v>0.8563</v>
       </c>
       <c r="Z2" s="5" t="n">
-        <v>0.2194</v>
+        <v>0.2497</v>
       </c>
       <c r="AA2" s="3" t="inlineStr">
         <is>
-          <t>results/synthetic/p53_additive_LINEAR/p53_additive_cv_loss_curves.png</t>
+          <t>results/synthetic/p53_epistatic_LINEAR/p53_epistatic_cv_loss_curves.png</t>
         </is>
       </c>
       <c r="AB2" s="3" t="inlineStr">
         <is>
-          <t>results/synthetic/p53_additive_LINEAR/p53_additive_predicted_vs_actual_test.png</t>
+          <t>results/synthetic/p53_epistatic_LINEAR/p53_epistatic_predicted_vs_actual_test.png</t>
         </is>
       </c>
       <c r="AC2" s="3" t="inlineStr">
         <is>
-          <t>results/synthetic/p53_additive_LINEAR/p53_additive_integrated_gradients_heatmap.png</t>
+          <t>results/synthetic/p53_epistatic_LINEAR/p53_epistatic_integrated_gradients_heatmap.png</t>
         </is>
       </c>
       <c r="AD2" s="3" t="inlineStr">
         <is>
-          <t>results/synthetic/p53_additive_LINEAR/p53_additive_integrated_gradients_analysis.png</t>
+          <t>results/synthetic/p53_epistatic_LINEAR/p53_epistatic_integrated_gradients_analysis.png</t>
         </is>
       </c>
       <c r="AE2" t="inlineStr">
         <is>
-          <t>First p53 after OOOM</t>
+          <t>p53 epistatic</t>
         </is>
       </c>
     </row>
@@ -3099,13 +3623,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE1"/>
+  <dimension ref="A1:AE2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -3298,211 +3822,142 @@
         </is>
       </c>
     </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:AE1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="7" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="45" customWidth="1" min="5" max="5"/>
-    <col width="45" customWidth="1" min="6" max="6"/>
-    <col width="45" customWidth="1" min="7" max="7"/>
-    <col width="45" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="20" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
-    <col width="12" customWidth="1" min="13" max="13"/>
-    <col width="8" customWidth="1" min="14" max="14"/>
-    <col width="12" customWidth="1" min="15" max="15"/>
-    <col width="10" customWidth="1" min="16" max="16"/>
-    <col width="12" customWidth="1" min="17" max="17"/>
-    <col width="14" customWidth="1" min="18" max="18"/>
-    <col width="16" customWidth="1" min="19" max="19"/>
-    <col width="14" customWidth="1" min="20" max="20"/>
-    <col width="20" customWidth="1" min="21" max="21"/>
-    <col width="18" customWidth="1" min="22" max="22"/>
-    <col width="18" customWidth="1" min="23" max="23"/>
-    <col width="10" customWidth="1" min="24" max="24"/>
-    <col width="15" customWidth="1" min="25" max="25"/>
-    <col width="16" customWidth="1" min="26" max="26"/>
-    <col width="20" customWidth="1" min="27" max="27"/>
-    <col width="22" customWidth="1" min="28" max="28"/>
-    <col width="18" customWidth="1" min="29" max="29"/>
-    <col width="18" customWidth="1" min="30" max="30"/>
-    <col width="40" customWidth="1" min="31" max="31"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Run #</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Timestamp</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Dataset</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Command</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Config (input)</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Config snapshot</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Results dir</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Run log</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>pooling_method</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>hidden_dims</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>dropout_rate</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>learning_rate</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>batch_size</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>epochs</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>min_epochs</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>patience</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>loss_type</t>
-        </is>
-      </c>
-      <c r="R1" s="1" t="inlineStr">
-        <is>
-          <t>normalization</t>
-        </is>
-      </c>
-      <c r="S1" s="1" t="inlineStr">
-        <is>
-          <t>CV mean val R²</t>
-        </is>
-      </c>
-      <c r="T1" s="1" t="inlineStr">
-        <is>
-          <t>CV std val R²</t>
-        </is>
-      </c>
-      <c r="U1" s="1" t="inlineStr">
-        <is>
-          <t>CV mean val Spearman</t>
-        </is>
-      </c>
-      <c r="V1" s="1" t="inlineStr">
-        <is>
-          <t>CV std val Spearman</t>
-        </is>
-      </c>
-      <c r="W1" s="1" t="inlineStr">
-        <is>
-          <t>CV avg best epoch</t>
-        </is>
-      </c>
-      <c r="X1" s="1" t="inlineStr">
-        <is>
-          <t>Test R²</t>
-        </is>
-      </c>
-      <c r="Y1" s="1" t="inlineStr">
-        <is>
-          <t>Test Pearson r</t>
-        </is>
-      </c>
-      <c r="Z1" s="1" t="inlineStr">
-        <is>
-          <t>Test Spearman ρ</t>
-        </is>
-      </c>
-      <c r="AA1" s="1" t="inlineStr">
-        <is>
-          <t>CV loss curves</t>
-        </is>
-      </c>
-      <c r="AB1" s="1" t="inlineStr">
-        <is>
-          <t>Test pred vs actual</t>
-        </is>
-      </c>
-      <c r="AC1" s="1" t="inlineStr">
-        <is>
-          <t>IG heatmap</t>
-        </is>
-      </c>
-      <c r="AD1" s="1" t="inlineStr">
-        <is>
-          <t>IG analysis</t>
-        </is>
-      </c>
-      <c r="AE1" s="1" t="inlineStr">
-        <is>
-          <t>Notes</t>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2026-04-12 17:34</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>p53_nonlinear</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>python scripts/run_integrated_gradients.py configs/synthetic/p53_nonlinear_config.yaml</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>configs/synthetic/p53_nonlinear_config.yaml</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/p53_nonlinear_LINEAR/p53_nonlinear_config_snapshot_20260412_095601.yaml</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>results/synthetic/p53_nonlinear_LINEAR</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/p53_nonlinear_LINEAR/p53_nonlinear_run_log_20260412_095601.txt</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>esm_attention</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>1024-512-256-128</t>
+        </is>
+      </c>
+      <c r="K2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0.0005</v>
+      </c>
+      <c r="M2" t="n">
+        <v>256</v>
+      </c>
+      <c r="N2" t="n">
+        <v>50</v>
+      </c>
+      <c r="O2" t="n">
+        <v>10</v>
+      </c>
+      <c r="P2" t="n">
+        <v>15</v>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>huber</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="S2" s="4" t="n">
+        <v>0.6383</v>
+      </c>
+      <c r="T2" t="n">
+        <v>0.0738</v>
+      </c>
+      <c r="U2" s="5" t="n">
+        <v>0.2118</v>
+      </c>
+      <c r="V2" t="n">
+        <v>0.0164</v>
+      </c>
+      <c r="W2" t="n">
+        <v>43.8</v>
+      </c>
+      <c r="X2" s="4" t="n">
+        <v>0.7762</v>
+      </c>
+      <c r="Y2" s="4" t="n">
+        <v>0.8819</v>
+      </c>
+      <c r="Z2" s="5" t="n">
+        <v>0.2073</v>
+      </c>
+      <c r="AA2" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/p53_nonlinear_LINEAR/p53_nonlinear_cv_loss_curves.png</t>
+        </is>
+      </c>
+      <c r="AB2" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/p53_nonlinear_LINEAR/p53_nonlinear_predicted_vs_actual_test.png</t>
+        </is>
+      </c>
+      <c r="AC2" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/p53_nonlinear_LINEAR/p53_nonlinear_integrated_gradients_heatmap.png</t>
+        </is>
+      </c>
+      <c r="AD2" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/p53_nonlinear_LINEAR/p53_nonlinear_integrated_gradients_analysis.png</t>
+        </is>
+      </c>
+      <c r="AE2" t="inlineStr">
+        <is>
+          <t>p53 nonlinear</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H2" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA2" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB2" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC2" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD2" r:id="rId6"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
updated tracket with initial T4 results
</commit_message>
<xml_diff>
--- a/experiment_tracker.xlsx
+++ b/experiment_tracker.xlsx
@@ -475,7 +475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE1"/>
+  <dimension ref="A1:AE2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -668,7 +668,137 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2026-04-15 13:45</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>T4Lysozyme_epistatic</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>python scripts/run_integrated_gradients.py configs/synthetic/T4Lysozyme_epistatic_config.yaml</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_epistatic_LINEAR/T4Lysozyme_epistatic_config_snapshot_20260414_191324.yaml</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_epistatic_LINEAR</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_epistatic_LINEAR/T4Lysozyme_epistatic_run_log_20260414_191324.txt</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>esm_attention</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>512-256-128-64</t>
+        </is>
+      </c>
+      <c r="K2" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0.0008</v>
+      </c>
+      <c r="M2" t="n">
+        <v>128</v>
+      </c>
+      <c r="N2" t="n">
+        <v>50</v>
+      </c>
+      <c r="O2" t="n">
+        <v>10</v>
+      </c>
+      <c r="P2" t="n">
+        <v>15</v>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>huber</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="S2" s="4" t="n">
+        <v>0.9171</v>
+      </c>
+      <c r="T2" t="n">
+        <v>0.0271</v>
+      </c>
+      <c r="U2" s="5" t="n">
+        <v>0.3681</v>
+      </c>
+      <c r="V2" t="n">
+        <v>0.0337</v>
+      </c>
+      <c r="W2" t="n">
+        <v>45.6</v>
+      </c>
+      <c r="X2" s="4" t="n">
+        <v>0.9371</v>
+      </c>
+      <c r="Y2" s="4" t="n">
+        <v>0.9684</v>
+      </c>
+      <c r="Z2" s="5" t="n">
+        <v>0.4195</v>
+      </c>
+      <c r="AA2" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_epistatic_LINEAR/T4Lysozyme_epistatic_cv_loss_curves.png</t>
+        </is>
+      </c>
+      <c r="AB2" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_epistatic_LINEAR/T4Lysozyme_epistatic_predicted_vs_actual_test.png</t>
+        </is>
+      </c>
+      <c r="AC2" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_epistatic_LINEAR/T4Lysozyme_epistatic_integrated_gradients_heatmap.png</t>
+        </is>
+      </c>
+      <c r="AD2" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_epistatic_LINEAR/T4Lysozyme_epistatic_integrated_gradients_analysis.png</t>
+        </is>
+      </c>
+      <c r="AE2" t="inlineStr">
+        <is>
+          <t>Rana: initial run</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H2" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA2" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB2" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC2" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD2" r:id="rId6"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -679,7 +809,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE1"/>
+  <dimension ref="A1:AE2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -872,7 +1002,138 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2026-04-15 13:45</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>T4Lysozyme_nonlinear</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>python scripts/run_integrated_gradients.py configs/synthetic/T4Lysozyme_nonlinear_config.yaml</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_nonlinear_LINEAR/T4Lysozyme_nonlinear_config_snapshot_20260414_201415.yaml</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_nonlinear_LINEAR</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_nonlinear_LINEAR/T4Lysozyme_nonlinear_run_log_20260414_201415.txt</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>esm_attention</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>512-256-128-64</t>
+        </is>
+      </c>
+      <c r="K2" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0.0008</v>
+      </c>
+      <c r="M2" t="n">
+        <v>128</v>
+      </c>
+      <c r="N2" t="n">
+        <v>50</v>
+      </c>
+      <c r="O2" t="n">
+        <v>10</v>
+      </c>
+      <c r="P2" t="n">
+        <v>15</v>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>huber</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="S2" s="4" t="n">
+        <v>0.9556</v>
+      </c>
+      <c r="T2" t="n">
+        <v>0.0211</v>
+      </c>
+      <c r="U2" s="5" t="n">
+        <v>0.4067</v>
+      </c>
+      <c r="V2" t="n">
+        <v>0.0898</v>
+      </c>
+      <c r="W2" t="n">
+        <v>37.4</v>
+      </c>
+      <c r="X2" s="4" t="n">
+        <v>0.9807</v>
+      </c>
+      <c r="Y2" s="4" t="n">
+        <v>0.991</v>
+      </c>
+      <c r="Z2" s="5" t="n">
+        <v>0.3861</v>
+      </c>
+      <c r="AA2" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_nonlinear_LINEAR/T4Lysozyme_nonlinear_cv_loss_curves.png</t>
+        </is>
+      </c>
+      <c r="AB2" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_nonlinear_LINEAR/T4Lysozyme_nonlinear_predicted_vs_actual_test.png</t>
+        </is>
+      </c>
+      <c r="AC2" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_nonlinear_LINEAR/T4Lysozyme_nonlinear_integrated_gradients_heatmap.png</t>
+        </is>
+      </c>
+      <c r="AD2" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_nonlinear_LINEAR/T4Lysozyme_nonlinear_integrated_gradients_analysis.png</t>
+        </is>
+      </c>
+      <c r="AE2" t="inlineStr">
+        <is>
+          <t>Rana: initial run</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H2" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA2" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB2" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC2" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD2" r:id="rId6"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1754,7 +2015,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1924,6 +2185,84 @@
       <c r="F6" t="inlineStr">
         <is>
           <t>results/synthetic/p53_nonlinear_LINEAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>T4Lysozyme_additive</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="n">
+        <v>0.8735000000000001</v>
+      </c>
+      <c r="C7" s="5" t="n">
+        <v>0.451</v>
+      </c>
+      <c r="D7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>2026-04-15 13:44</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_additive_LINEAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>T4Lysozyme_epistatic</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="n">
+        <v>0.9371</v>
+      </c>
+      <c r="C8" s="5" t="n">
+        <v>0.4195</v>
+      </c>
+      <c r="D8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>2026-04-15 13:45</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_epistatic_LINEAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>T4Lysozyme_nonlinear</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="n">
+        <v>0.9807</v>
+      </c>
+      <c r="C9" s="5" t="n">
+        <v>0.3861</v>
+      </c>
+      <c r="D9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>2026-04-15 13:45</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_nonlinear_LINEAR</t>
         </is>
       </c>
     </row>
@@ -3968,7 +4307,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE1"/>
+  <dimension ref="A1:AE2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -4161,7 +4500,137 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2026-04-15 13:44</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>T4Lysozyme_additive</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>python scripts/run_integrated_gradients.py configs/synthetic/T4Lysozyme_additive_config.yaml</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_additive_LINEAR/T4Lysozyme_additive_config_snapshot_20260414_173426.yaml</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_additive_LINEAR</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_additive_LINEAR/T4Lysozyme_additive_run_log_20260414_173426.txt</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>esm_attention</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>512-256-128-64</t>
+        </is>
+      </c>
+      <c r="K2" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0.0008</v>
+      </c>
+      <c r="M2" t="n">
+        <v>128</v>
+      </c>
+      <c r="N2" t="n">
+        <v>50</v>
+      </c>
+      <c r="O2" t="n">
+        <v>10</v>
+      </c>
+      <c r="P2" t="n">
+        <v>15</v>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>huber</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="S2" s="4" t="n">
+        <v>0.9273</v>
+      </c>
+      <c r="T2" t="n">
+        <v>0.0244</v>
+      </c>
+      <c r="U2" s="5" t="n">
+        <v>0.3816</v>
+      </c>
+      <c r="V2" t="n">
+        <v>0.0864</v>
+      </c>
+      <c r="W2" t="n">
+        <v>45.4</v>
+      </c>
+      <c r="X2" s="4" t="n">
+        <v>0.8735000000000001</v>
+      </c>
+      <c r="Y2" s="4" t="n">
+        <v>0.9350000000000001</v>
+      </c>
+      <c r="Z2" s="5" t="n">
+        <v>0.451</v>
+      </c>
+      <c r="AA2" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_additive_LINEAR/T4Lysozyme_additive_cv_loss_curves.png</t>
+        </is>
+      </c>
+      <c r="AB2" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_additive_LINEAR/T4Lysozyme_additive_predicted_vs_actual_test.png</t>
+        </is>
+      </c>
+      <c r="AC2" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_additive_LINEAR/T4Lysozyme_additive_integrated_gradients_heatmap.png</t>
+        </is>
+      </c>
+      <c r="AD2" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_additive_LINEAR/T4Lysozyme_additive_integrated_gradients_analysis.png</t>
+        </is>
+      </c>
+      <c r="AE2" t="inlineStr">
+        <is>
+          <t>Rana: initial run</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H2" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA2" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB2" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC2" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD2" r:id="rId6"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
More rows for p53
</commit_message>
<xml_diff>
--- a/experiment_tracker.xlsx
+++ b/experiment_tracker.xlsx
@@ -1862,7 +1862,7 @@
         <v>0.2194</v>
       </c>
       <c r="D4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -1888,7 +1888,7 @@
         <v>0.2497</v>
       </c>
       <c r="D5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -1914,7 +1914,7 @@
         <v>0.2073</v>
       </c>
       <c r="D6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -2818,6 +2818,611 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:AE4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="7" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="45" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="45" customWidth="1" min="7" max="7"/>
+    <col width="45" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="8" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
+    <col width="10" customWidth="1" min="16" max="16"/>
+    <col width="12" customWidth="1" min="17" max="17"/>
+    <col width="14" customWidth="1" min="18" max="18"/>
+    <col width="16" customWidth="1" min="19" max="19"/>
+    <col width="14" customWidth="1" min="20" max="20"/>
+    <col width="20" customWidth="1" min="21" max="21"/>
+    <col width="18" customWidth="1" min="22" max="22"/>
+    <col width="18" customWidth="1" min="23" max="23"/>
+    <col width="10" customWidth="1" min="24" max="24"/>
+    <col width="15" customWidth="1" min="25" max="25"/>
+    <col width="16" customWidth="1" min="26" max="26"/>
+    <col width="20" customWidth="1" min="27" max="27"/>
+    <col width="22" customWidth="1" min="28" max="28"/>
+    <col width="18" customWidth="1" min="29" max="29"/>
+    <col width="18" customWidth="1" min="30" max="30"/>
+    <col width="40" customWidth="1" min="31" max="31"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Run #</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Timestamp</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Dataset</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Command</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Config (input)</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Config snapshot</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Results dir</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Run log</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>pooling_method</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>hidden_dims</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>dropout_rate</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>learning_rate</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>batch_size</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>epochs</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>min_epochs</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>patience</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>loss_type</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>normalization</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>CV mean val R²</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>CV std val R²</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>CV mean val Spearman</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>CV std val Spearman</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>CV avg best epoch</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>Test R²</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>Test Pearson r</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>Test Spearman ρ</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>CV loss curves</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>Test pred vs actual</t>
+        </is>
+      </c>
+      <c r="AC1" s="1" t="inlineStr">
+        <is>
+          <t>IG heatmap</t>
+        </is>
+      </c>
+      <c r="AD1" s="1" t="inlineStr">
+        <is>
+          <t>IG analysis</t>
+        </is>
+      </c>
+      <c r="AE1" s="1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2026-04-12 09:15</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>p53_additive</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>python scripts/run_integrated_gradients.py configs/synthetic/p53_additive_config.yaml</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>configs/synthetic/p53_additive_config.yaml</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/p53_additive_LINEAR/p53_additive_config_snapshot_20260412_012304.yaml</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>results/synthetic/p53_additive_LINEAR</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/p53_additive_LINEAR/p53_additive_run_log_20260412_012304.txt</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>esm_attention</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>1024-512-256-128</t>
+        </is>
+      </c>
+      <c r="K2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0.0005</v>
+      </c>
+      <c r="M2" t="n">
+        <v>256</v>
+      </c>
+      <c r="N2" t="n">
+        <v>50</v>
+      </c>
+      <c r="O2" t="n">
+        <v>10</v>
+      </c>
+      <c r="P2" t="n">
+        <v>15</v>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>huber</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="S2" s="4" t="n">
+        <v>0.6383</v>
+      </c>
+      <c r="T2" t="n">
+        <v>0.0736</v>
+      </c>
+      <c r="U2" s="5" t="n">
+        <v>0.2053</v>
+      </c>
+      <c r="V2" t="n">
+        <v>0.0231</v>
+      </c>
+      <c r="W2" t="n">
+        <v>47.6</v>
+      </c>
+      <c r="X2" s="4" t="n">
+        <v>0.7309</v>
+      </c>
+      <c r="Y2" s="4" t="n">
+        <v>0.8561</v>
+      </c>
+      <c r="Z2" s="5" t="n">
+        <v>0.2194</v>
+      </c>
+      <c r="AA2" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/p53_additive_LINEAR/p53_additive_cv_loss_curves.png</t>
+        </is>
+      </c>
+      <c r="AB2" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/p53_additive_LINEAR/p53_additive_predicted_vs_actual_test.png</t>
+        </is>
+      </c>
+      <c r="AC2" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/p53_additive_LINEAR/p53_additive_integrated_gradients_heatmap.png</t>
+        </is>
+      </c>
+      <c r="AD2" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/p53_additive_LINEAR/p53_additive_integrated_gradients_analysis.png</t>
+        </is>
+      </c>
+      <c r="AE2" t="inlineStr">
+        <is>
+          <t>First p53 after OOOM</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-04-12 17:28</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>p53_additive</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>python scripts/run_integrated_gradients.py configs/synthetic/p53_additive_config.yaml</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>configs/synthetic/p53_additive_config.yaml</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/p53_additive_LINEAR/p53_additive_config_snapshot_20260412_140326.yaml</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>results/synthetic/p53_additive_LINEAR</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/p53_additive_LINEAR/p53_additive_run_log_20260412_140326.txt</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>esm_attention</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>2056-1024-512-256</t>
+        </is>
+      </c>
+      <c r="K3" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0.0005</v>
+      </c>
+      <c r="M3" t="n">
+        <v>256</v>
+      </c>
+      <c r="N3" t="n">
+        <v>50</v>
+      </c>
+      <c r="O3" t="n">
+        <v>15</v>
+      </c>
+      <c r="P3" t="n">
+        <v>30</v>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>huber</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="S3" s="4" t="n">
+        <v>0.5503</v>
+      </c>
+      <c r="T3" t="n">
+        <v>0.1706</v>
+      </c>
+      <c r="U3" s="5" t="n">
+        <v>0.2316</v>
+      </c>
+      <c r="V3" t="n">
+        <v>0.0728</v>
+      </c>
+      <c r="W3" t="n">
+        <v>46.6</v>
+      </c>
+      <c r="X3" s="4" t="n">
+        <v>0.6378</v>
+      </c>
+      <c r="Y3" s="4" t="n">
+        <v>0.8038</v>
+      </c>
+      <c r="Z3" s="2" t="n">
+        <v>0.1813</v>
+      </c>
+      <c r="AA3" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/p53_additive_LINEAR/p53_additive_cv_loss_curves.png</t>
+        </is>
+      </c>
+      <c r="AB3" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/p53_additive_LINEAR/p53_additive_predicted_vs_actual_test.png</t>
+        </is>
+      </c>
+      <c r="AC3" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/p53_additive_LINEAR/p53_additive_integrated_gradients_heatmap.png</t>
+        </is>
+      </c>
+      <c r="AD3" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/p53_additive_LINEAR/p53_additive_integrated_gradients_analysis.png</t>
+        </is>
+      </c>
+      <c r="AE3" t="inlineStr">
+        <is>
+          <t>p53 additive 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-04-15 12:25</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>p53_additive</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>python scripts/run_integrated_gradients.py configs/synthetic/p53_additive_config.yaml</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>configs/synthetic/p53_additive_config.yaml</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/p53_additive_LINEAR/p53_additive_config_snapshot_20260414_113226.yaml</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>results/synthetic/p53_additive_LINEAR</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/p53_additive_LINEAR/p53_additive_run_log_20260414_113226.txt</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>esm_attention</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>518-256-128-64</t>
+        </is>
+      </c>
+      <c r="K4" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0.0005</v>
+      </c>
+      <c r="M4" t="n">
+        <v>256</v>
+      </c>
+      <c r="N4" t="n">
+        <v>50</v>
+      </c>
+      <c r="O4" t="n">
+        <v>10</v>
+      </c>
+      <c r="P4" t="n">
+        <v>15</v>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>huber</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="S4" s="4" t="n">
+        <v>0.6342</v>
+      </c>
+      <c r="T4" t="n">
+        <v>0.0704</v>
+      </c>
+      <c r="U4" s="5" t="n">
+        <v>0.2099</v>
+      </c>
+      <c r="V4" t="n">
+        <v>0.0283</v>
+      </c>
+      <c r="W4" t="n">
+        <v>44</v>
+      </c>
+      <c r="X4" s="4" t="n">
+        <v>0.7203000000000001</v>
+      </c>
+      <c r="Y4" s="4" t="n">
+        <v>0.8514</v>
+      </c>
+      <c r="Z4" s="2" t="n">
+        <v>0.1887</v>
+      </c>
+      <c r="AA4" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/p53_additive_LINEAR/p53_additive_cv_loss_curves.png</t>
+        </is>
+      </c>
+      <c r="AB4" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/p53_additive_LINEAR/p53_additive_predicted_vs_actual_test.png</t>
+        </is>
+      </c>
+      <c r="AC4" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/p53_additive_LINEAR/p53_additive_integrated_gradients_heatmap.png</t>
+        </is>
+      </c>
+      <c r="AD4" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/p53_additive_LINEAR/p53_additive_integrated_gradients_analysis.png</t>
+        </is>
+      </c>
+      <c r="AE4" t="inlineStr">
+        <is>
+          <t>p53 additive with 512 dimensions</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H2" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA2" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB2" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC2" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD2" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F3" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H3" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA3" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB3" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC3" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD3" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F4" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H4" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA4" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB4" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC4" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD4" r:id="rId18"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:AE3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -3017,37 +3622,37 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-04-12 09:15</t>
+          <t>2026-04-12 17:34</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>p53_additive</t>
+          <t>p53_epistatic</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>python scripts/run_integrated_gradients.py configs/synthetic/p53_additive_config.yaml</t>
+          <t>python scripts/run_integrated_gradients.py configs/synthetic/p53_epistatic_config.yaml</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>configs/synthetic/p53_additive_config.yaml</t>
+          <t>configs/synthetic/p53_epistatic_config.yaml</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>results/synthetic/p53_additive_LINEAR/p53_additive_config_snapshot_20260412_012304.yaml</t>
+          <t>results/synthetic/p53_epistatic_LINEAR/p53_epistatic_config_snapshot_20260412_095552.yaml</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>results/synthetic/p53_additive_LINEAR</t>
+          <t>results/synthetic/p53_epistatic_LINEAR</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>results/synthetic/p53_additive_LINEAR/p53_additive_run_log_20260412_012304.txt</t>
+          <t>results/synthetic/p53_epistatic_LINEAR/p53_epistatic_run_log_20260412_095552.txt</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -3089,52 +3694,52 @@
         </is>
       </c>
       <c r="S2" s="4" t="n">
-        <v>0.6383</v>
+        <v>0.5198</v>
       </c>
       <c r="T2" t="n">
-        <v>0.0736</v>
+        <v>0.1104</v>
       </c>
       <c r="U2" s="5" t="n">
-        <v>0.2053</v>
+        <v>0.2172</v>
       </c>
       <c r="V2" t="n">
-        <v>0.0231</v>
+        <v>0.0433</v>
       </c>
       <c r="W2" t="n">
-        <v>47.6</v>
+        <v>45.2</v>
       </c>
       <c r="X2" s="4" t="n">
-        <v>0.7309</v>
+        <v>0.7277</v>
       </c>
       <c r="Y2" s="4" t="n">
-        <v>0.8561</v>
+        <v>0.8563</v>
       </c>
       <c r="Z2" s="5" t="n">
-        <v>0.2194</v>
+        <v>0.2497</v>
       </c>
       <c r="AA2" s="3" t="inlineStr">
         <is>
-          <t>results/synthetic/p53_additive_LINEAR/p53_additive_cv_loss_curves.png</t>
+          <t>results/synthetic/p53_epistatic_LINEAR/p53_epistatic_cv_loss_curves.png</t>
         </is>
       </c>
       <c r="AB2" s="3" t="inlineStr">
         <is>
-          <t>results/synthetic/p53_additive_LINEAR/p53_additive_predicted_vs_actual_test.png</t>
+          <t>results/synthetic/p53_epistatic_LINEAR/p53_epistatic_predicted_vs_actual_test.png</t>
         </is>
       </c>
       <c r="AC2" s="3" t="inlineStr">
         <is>
-          <t>results/synthetic/p53_additive_LINEAR/p53_additive_integrated_gradients_heatmap.png</t>
+          <t>results/synthetic/p53_epistatic_LINEAR/p53_epistatic_integrated_gradients_heatmap.png</t>
         </is>
       </c>
       <c r="AD2" s="3" t="inlineStr">
         <is>
-          <t>results/synthetic/p53_additive_LINEAR/p53_additive_integrated_gradients_analysis.png</t>
+          <t>results/synthetic/p53_epistatic_LINEAR/p53_epistatic_integrated_gradients_analysis.png</t>
         </is>
       </c>
       <c r="AE2" t="inlineStr">
         <is>
-          <t>First p53 after OOOM</t>
+          <t>p53 epistatic</t>
         </is>
       </c>
     </row>
@@ -3144,37 +3749,37 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-04-12 17:28</t>
+          <t>2026-04-15 12:24</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>p53_additive</t>
+          <t>p53_epistatic</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>python scripts/run_integrated_gradients.py configs/synthetic/p53_additive_config.yaml</t>
+          <t>python scripts/run_integrated_gradients.py configs/synthetic/p53_epistatic_config.yaml</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>configs/synthetic/p53_additive_config.yaml</t>
+          <t>configs/synthetic/p53_epistatic_config.yaml</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>results/synthetic/p53_additive_LINEAR/p53_additive_config_snapshot_20260412_140326.yaml</t>
+          <t>results/synthetic/p53_epistatic_LINEAR/p53_epistatic_config_snapshot_20260414_113603.yaml</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>results/synthetic/p53_additive_LINEAR</t>
+          <t>results/synthetic/p53_epistatic_LINEAR</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>results/synthetic/p53_additive_LINEAR/p53_additive_run_log_20260412_140326.txt</t>
+          <t>results/synthetic/p53_epistatic_LINEAR/p53_epistatic_run_log_20260414_113602.txt</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -3184,7 +3789,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2056-1024-512-256</t>
+          <t>512-256-128-64</t>
         </is>
       </c>
       <c r="K3" t="n">
@@ -3200,7 +3805,7 @@
         <v>50</v>
       </c>
       <c r="O3" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="P3" t="n">
         <v>30</v>
@@ -3216,52 +3821,52 @@
         </is>
       </c>
       <c r="S3" s="4" t="n">
-        <v>0.5503</v>
+        <v>0.5796</v>
       </c>
       <c r="T3" t="n">
-        <v>0.1706</v>
+        <v>0.1067</v>
       </c>
       <c r="U3" s="5" t="n">
-        <v>0.2316</v>
+        <v>0.2095</v>
       </c>
       <c r="V3" t="n">
-        <v>0.0728</v>
+        <v>0.0449</v>
       </c>
       <c r="W3" t="n">
-        <v>46.6</v>
+        <v>45.6</v>
       </c>
       <c r="X3" s="4" t="n">
-        <v>0.6378</v>
+        <v>0.7165</v>
       </c>
       <c r="Y3" s="4" t="n">
-        <v>0.8038</v>
-      </c>
-      <c r="Z3" s="2" t="n">
-        <v>0.1813</v>
+        <v>0.8471</v>
+      </c>
+      <c r="Z3" s="5" t="n">
+        <v>0.2336</v>
       </c>
       <c r="AA3" s="3" t="inlineStr">
         <is>
-          <t>results/synthetic/p53_additive_LINEAR/p53_additive_cv_loss_curves.png</t>
+          <t>results/synthetic/p53_epistatic_LINEAR/p53_epistatic_cv_loss_curves.png</t>
         </is>
       </c>
       <c r="AB3" s="3" t="inlineStr">
         <is>
-          <t>results/synthetic/p53_additive_LINEAR/p53_additive_predicted_vs_actual_test.png</t>
+          <t>results/synthetic/p53_epistatic_LINEAR/p53_epistatic_predicted_vs_actual_test.png</t>
         </is>
       </c>
       <c r="AC3" s="3" t="inlineStr">
         <is>
-          <t>results/synthetic/p53_additive_LINEAR/p53_additive_integrated_gradients_heatmap.png</t>
+          <t>results/synthetic/p53_epistatic_LINEAR/p53_epistatic_integrated_gradients_heatmap.png</t>
         </is>
       </c>
       <c r="AD3" s="3" t="inlineStr">
         <is>
-          <t>results/synthetic/p53_additive_LINEAR/p53_additive_integrated_gradients_analysis.png</t>
+          <t>results/synthetic/p53_epistatic_LINEAR/p53_epistatic_integrated_gradients_analysis.png</t>
         </is>
       </c>
       <c r="AE3" t="inlineStr">
         <is>
-          <t>p53 additive 2</t>
+          <t>p53 epistatic with 512 dimensions</t>
         </is>
       </c>
     </row>
@@ -3284,13 +3889,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE2"/>
+  <dimension ref="A1:AE3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -3494,32 +4099,32 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>p53_epistatic</t>
+          <t>p53_nonlinear</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>python scripts/run_integrated_gradients.py configs/synthetic/p53_epistatic_config.yaml</t>
+          <t>python scripts/run_integrated_gradients.py configs/synthetic/p53_nonlinear_config.yaml</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>configs/synthetic/p53_epistatic_config.yaml</t>
+          <t>configs/synthetic/p53_nonlinear_config.yaml</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>results/synthetic/p53_epistatic_LINEAR/p53_epistatic_config_snapshot_20260412_095552.yaml</t>
+          <t>results/synthetic/p53_nonlinear_LINEAR/p53_nonlinear_config_snapshot_20260412_095601.yaml</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>results/synthetic/p53_epistatic_LINEAR</t>
+          <t>results/synthetic/p53_nonlinear_LINEAR</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>results/synthetic/p53_epistatic_LINEAR/p53_epistatic_run_log_20260412_095552.txt</t>
+          <t>results/synthetic/p53_nonlinear_LINEAR/p53_nonlinear_run_log_20260412_095601.txt</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -3561,52 +4166,179 @@
         </is>
       </c>
       <c r="S2" s="4" t="n">
-        <v>0.5198</v>
+        <v>0.6383</v>
       </c>
       <c r="T2" t="n">
-        <v>0.1104</v>
+        <v>0.0738</v>
       </c>
       <c r="U2" s="5" t="n">
-        <v>0.2172</v>
+        <v>0.2118</v>
       </c>
       <c r="V2" t="n">
-        <v>0.0433</v>
+        <v>0.0164</v>
       </c>
       <c r="W2" t="n">
-        <v>45.2</v>
+        <v>43.8</v>
       </c>
       <c r="X2" s="4" t="n">
-        <v>0.7277</v>
+        <v>0.7762</v>
       </c>
       <c r="Y2" s="4" t="n">
-        <v>0.8563</v>
+        <v>0.8819</v>
       </c>
       <c r="Z2" s="5" t="n">
-        <v>0.2497</v>
+        <v>0.2073</v>
       </c>
       <c r="AA2" s="3" t="inlineStr">
         <is>
-          <t>results/synthetic/p53_epistatic_LINEAR/p53_epistatic_cv_loss_curves.png</t>
+          <t>results/synthetic/p53_nonlinear_LINEAR/p53_nonlinear_cv_loss_curves.png</t>
         </is>
       </c>
       <c r="AB2" s="3" t="inlineStr">
         <is>
-          <t>results/synthetic/p53_epistatic_LINEAR/p53_epistatic_predicted_vs_actual_test.png</t>
+          <t>results/synthetic/p53_nonlinear_LINEAR/p53_nonlinear_predicted_vs_actual_test.png</t>
         </is>
       </c>
       <c r="AC2" s="3" t="inlineStr">
         <is>
-          <t>results/synthetic/p53_epistatic_LINEAR/p53_epistatic_integrated_gradients_heatmap.png</t>
+          <t>results/synthetic/p53_nonlinear_LINEAR/p53_nonlinear_integrated_gradients_heatmap.png</t>
         </is>
       </c>
       <c r="AD2" s="3" t="inlineStr">
         <is>
-          <t>results/synthetic/p53_epistatic_LINEAR/p53_epistatic_integrated_gradients_analysis.png</t>
+          <t>results/synthetic/p53_nonlinear_LINEAR/p53_nonlinear_integrated_gradients_analysis.png</t>
         </is>
       </c>
       <c r="AE2" t="inlineStr">
         <is>
-          <t>p53 epistatic</t>
+          <t>p53 nonlinear</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-04-15 12:24</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>p53_nonlinear</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>python scripts/run_integrated_gradients.py configs/synthetic/p53_nonlinear_config.yaml</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>configs/synthetic/p53_nonlinear_config.yaml</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/p53_nonlinear_LINEAR/p53_nonlinear_config_snapshot_20260414_114421.yaml</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>results/synthetic/p53_nonlinear_LINEAR</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/p53_nonlinear_LINEAR/p53_nonlinear_run_log_20260414_114421.txt</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>esm_attention</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>512-256-128-64</t>
+        </is>
+      </c>
+      <c r="K3" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0.0005</v>
+      </c>
+      <c r="M3" t="n">
+        <v>256</v>
+      </c>
+      <c r="N3" t="n">
+        <v>50</v>
+      </c>
+      <c r="O3" t="n">
+        <v>20</v>
+      </c>
+      <c r="P3" t="n">
+        <v>30</v>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>huber</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="S3" s="4" t="n">
+        <v>0.6254999999999999</v>
+      </c>
+      <c r="T3" t="n">
+        <v>0.0738</v>
+      </c>
+      <c r="U3" s="5" t="n">
+        <v>0.229</v>
+      </c>
+      <c r="V3" t="n">
+        <v>0.0224</v>
+      </c>
+      <c r="W3" t="n">
+        <v>46.4</v>
+      </c>
+      <c r="X3" s="4" t="n">
+        <v>0.7698</v>
+      </c>
+      <c r="Y3" s="4" t="n">
+        <v>0.8784999999999999</v>
+      </c>
+      <c r="Z3" s="2" t="n">
+        <v>0.1736</v>
+      </c>
+      <c r="AA3" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/p53_nonlinear_LINEAR/p53_nonlinear_cv_loss_curves.png</t>
+        </is>
+      </c>
+      <c r="AB3" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/p53_nonlinear_LINEAR/p53_nonlinear_predicted_vs_actual_test.png</t>
+        </is>
+      </c>
+      <c r="AC3" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/p53_nonlinear_LINEAR/p53_nonlinear_integrated_gradients_heatmap.png</t>
+        </is>
+      </c>
+      <c r="AD3" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/p53_nonlinear_LINEAR/p53_nonlinear_integrated_gradients_analysis.png</t>
+        </is>
+      </c>
+      <c r="AE3" t="inlineStr">
+        <is>
+          <t>p53 nonlinear with 512 dimensions</t>
         </is>
       </c>
     </row>
@@ -3618,345 +4350,12 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB2" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC2" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD2" r:id="rId6"/>
-  </hyperlinks>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:AE2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="7" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="45" customWidth="1" min="5" max="5"/>
-    <col width="45" customWidth="1" min="6" max="6"/>
-    <col width="45" customWidth="1" min="7" max="7"/>
-    <col width="45" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="20" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
-    <col width="12" customWidth="1" min="13" max="13"/>
-    <col width="8" customWidth="1" min="14" max="14"/>
-    <col width="12" customWidth="1" min="15" max="15"/>
-    <col width="10" customWidth="1" min="16" max="16"/>
-    <col width="12" customWidth="1" min="17" max="17"/>
-    <col width="14" customWidth="1" min="18" max="18"/>
-    <col width="16" customWidth="1" min="19" max="19"/>
-    <col width="14" customWidth="1" min="20" max="20"/>
-    <col width="20" customWidth="1" min="21" max="21"/>
-    <col width="18" customWidth="1" min="22" max="22"/>
-    <col width="18" customWidth="1" min="23" max="23"/>
-    <col width="10" customWidth="1" min="24" max="24"/>
-    <col width="15" customWidth="1" min="25" max="25"/>
-    <col width="16" customWidth="1" min="26" max="26"/>
-    <col width="20" customWidth="1" min="27" max="27"/>
-    <col width="22" customWidth="1" min="28" max="28"/>
-    <col width="18" customWidth="1" min="29" max="29"/>
-    <col width="18" customWidth="1" min="30" max="30"/>
-    <col width="40" customWidth="1" min="31" max="31"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Run #</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Timestamp</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Dataset</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Command</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Config (input)</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Config snapshot</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Results dir</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Run log</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>pooling_method</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>hidden_dims</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>dropout_rate</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>learning_rate</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>batch_size</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>epochs</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>min_epochs</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>patience</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>loss_type</t>
-        </is>
-      </c>
-      <c r="R1" s="1" t="inlineStr">
-        <is>
-          <t>normalization</t>
-        </is>
-      </c>
-      <c r="S1" s="1" t="inlineStr">
-        <is>
-          <t>CV mean val R²</t>
-        </is>
-      </c>
-      <c r="T1" s="1" t="inlineStr">
-        <is>
-          <t>CV std val R²</t>
-        </is>
-      </c>
-      <c r="U1" s="1" t="inlineStr">
-        <is>
-          <t>CV mean val Spearman</t>
-        </is>
-      </c>
-      <c r="V1" s="1" t="inlineStr">
-        <is>
-          <t>CV std val Spearman</t>
-        </is>
-      </c>
-      <c r="W1" s="1" t="inlineStr">
-        <is>
-          <t>CV avg best epoch</t>
-        </is>
-      </c>
-      <c r="X1" s="1" t="inlineStr">
-        <is>
-          <t>Test R²</t>
-        </is>
-      </c>
-      <c r="Y1" s="1" t="inlineStr">
-        <is>
-          <t>Test Pearson r</t>
-        </is>
-      </c>
-      <c r="Z1" s="1" t="inlineStr">
-        <is>
-          <t>Test Spearman ρ</t>
-        </is>
-      </c>
-      <c r="AA1" s="1" t="inlineStr">
-        <is>
-          <t>CV loss curves</t>
-        </is>
-      </c>
-      <c r="AB1" s="1" t="inlineStr">
-        <is>
-          <t>Test pred vs actual</t>
-        </is>
-      </c>
-      <c r="AC1" s="1" t="inlineStr">
-        <is>
-          <t>IG heatmap</t>
-        </is>
-      </c>
-      <c r="AD1" s="1" t="inlineStr">
-        <is>
-          <t>IG analysis</t>
-        </is>
-      </c>
-      <c r="AE1" s="1" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>2026-04-12 17:34</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>p53_nonlinear</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>python scripts/run_integrated_gradients.py configs/synthetic/p53_nonlinear_config.yaml</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>configs/synthetic/p53_nonlinear_config.yaml</t>
-        </is>
-      </c>
-      <c r="F2" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/p53_nonlinear_LINEAR/p53_nonlinear_config_snapshot_20260412_095601.yaml</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>results/synthetic/p53_nonlinear_LINEAR</t>
-        </is>
-      </c>
-      <c r="H2" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/p53_nonlinear_LINEAR/p53_nonlinear_run_log_20260412_095601.txt</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>esm_attention</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>1024-512-256-128</t>
-        </is>
-      </c>
-      <c r="K2" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="L2" t="n">
-        <v>0.0005</v>
-      </c>
-      <c r="M2" t="n">
-        <v>256</v>
-      </c>
-      <c r="N2" t="n">
-        <v>50</v>
-      </c>
-      <c r="O2" t="n">
-        <v>10</v>
-      </c>
-      <c r="P2" t="n">
-        <v>15</v>
-      </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>huber</t>
-        </is>
-      </c>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="S2" s="4" t="n">
-        <v>0.6383</v>
-      </c>
-      <c r="T2" t="n">
-        <v>0.0738</v>
-      </c>
-      <c r="U2" s="5" t="n">
-        <v>0.2118</v>
-      </c>
-      <c r="V2" t="n">
-        <v>0.0164</v>
-      </c>
-      <c r="W2" t="n">
-        <v>43.8</v>
-      </c>
-      <c r="X2" s="4" t="n">
-        <v>0.7762</v>
-      </c>
-      <c r="Y2" s="4" t="n">
-        <v>0.8819</v>
-      </c>
-      <c r="Z2" s="5" t="n">
-        <v>0.2073</v>
-      </c>
-      <c r="AA2" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/p53_nonlinear_LINEAR/p53_nonlinear_cv_loss_curves.png</t>
-        </is>
-      </c>
-      <c r="AB2" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/p53_nonlinear_LINEAR/p53_nonlinear_predicted_vs_actual_test.png</t>
-        </is>
-      </c>
-      <c r="AC2" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/p53_nonlinear_LINEAR/p53_nonlinear_integrated_gradients_heatmap.png</t>
-        </is>
-      </c>
-      <c r="AD2" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/p53_nonlinear_LINEAR/p53_nonlinear_integrated_gradients_analysis.png</t>
-        </is>
-      </c>
-      <c r="AE2" t="inlineStr">
-        <is>
-          <t>p53 nonlinear</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H2" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA2" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB2" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC2" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD2" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F3" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H3" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA3" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB3" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC3" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD3" r:id="rId12"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add T4 run outputs and tracker updates for 12 runs
</commit_message>
<xml_diff>
--- a/experiment_tracker.xlsx
+++ b/experiment_tracker.xlsx
@@ -475,7 +475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE2"/>
+  <dimension ref="A1:AE6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -790,6 +790,514 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-04-15 16:16</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>T4Lysozyme_epistatic</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>python scripts/run_integrated_gradients.py configs/synthetic/T4Lysozyme_epistatic_config.yaml</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>configs/synthetic/T4Lysozyme_epistatic_config.yaml</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_epistatic_LINEAR/T4Lysozyme_epistatic_config_snapshot_20260415_142055.yaml</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_epistatic_LINEAR</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_epistatic_LINEAR/T4Lysozyme_epistatic_run_log_20260415_142055.txt</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>esm_attention</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>512-256-128-64</t>
+        </is>
+      </c>
+      <c r="K3" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0.0005999999999999999</v>
+      </c>
+      <c r="M3" t="n">
+        <v>128</v>
+      </c>
+      <c r="N3" t="n">
+        <v>80</v>
+      </c>
+      <c r="O3" t="n">
+        <v>15</v>
+      </c>
+      <c r="P3" t="n">
+        <v>20</v>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>huber</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="S3" t="n">
+        <v>0.9323</v>
+      </c>
+      <c r="T3" t="n">
+        <v>0.0329</v>
+      </c>
+      <c r="U3" t="n">
+        <v>0.4764</v>
+      </c>
+      <c r="V3" t="n">
+        <v>0.038</v>
+      </c>
+      <c r="W3" t="n">
+        <v>56.8</v>
+      </c>
+      <c r="X3" t="n">
+        <v>0.8976</v>
+      </c>
+      <c r="Y3" t="n">
+        <v>0.9477</v>
+      </c>
+      <c r="Z3" t="n">
+        <v>0.4264</v>
+      </c>
+      <c r="AA3" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_epistatic_LINEAR/T4Lysozyme_epistatic_cv_loss_curves.png</t>
+        </is>
+      </c>
+      <c r="AB3" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_epistatic_LINEAR/T4Lysozyme_epistatic_predicted_vs_actual_test.png</t>
+        </is>
+      </c>
+      <c r="AC3" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_epistatic_LINEAR/T4Lysozyme_epistatic_integrated_gradients_heatmap.png</t>
+        </is>
+      </c>
+      <c r="AD3" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_epistatic_LINEAR/T4Lysozyme_epistatic_integrated_gradients_analysis.png</t>
+        </is>
+      </c>
+      <c r="AE3" t="inlineStr">
+        <is>
+          <t>T4Lysozyme epistatic retune from baseline: dropout 0.4-&gt;0.35, learning_rate 8e-4-&gt;6e-4, epochs 50-&gt;80, patience 15-&gt;20, min_epochs 10-&gt;15; hidden dims unchanged (512-256-128-64).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-04-15 20:15</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>T4Lysozyme_epistatic</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>python scripts/run_integrated_gradients.py configs/synthetic/t4_tuning/T4Lysozyme_epistatic_E1_config.yaml</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>configs/synthetic/t4_tuning/T4Lysozyme_epistatic_E1_config.yaml</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_epistatic_LINEAR_E1/T4Lysozyme_epistatic_config_snapshot_20260415_194052.yaml</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_epistatic_LINEAR_E1</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_epistatic_LINEAR_E1/T4Lysozyme_epistatic_run_log_20260415_194052.txt</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>esm_attention</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>512-256-128-64</t>
+        </is>
+      </c>
+      <c r="K4" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0.0007</v>
+      </c>
+      <c r="M4" t="n">
+        <v>128</v>
+      </c>
+      <c r="N4" t="n">
+        <v>65</v>
+      </c>
+      <c r="O4" t="n">
+        <v>12</v>
+      </c>
+      <c r="P4" t="n">
+        <v>17</v>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>huber</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="S4" t="n">
+        <v>0.947</v>
+      </c>
+      <c r="T4" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="U4" t="n">
+        <v>0.5128</v>
+      </c>
+      <c r="V4" t="n">
+        <v>0.06469999999999999</v>
+      </c>
+      <c r="W4" t="n">
+        <v>47</v>
+      </c>
+      <c r="X4" t="n">
+        <v>0.9529</v>
+      </c>
+      <c r="Y4" t="n">
+        <v>0.9778</v>
+      </c>
+      <c r="Z4" t="n">
+        <v>0.4261</v>
+      </c>
+      <c r="AA4" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_epistatic_LINEAR_E1/T4Lysozyme_epistatic_cv_loss_curves.png</t>
+        </is>
+      </c>
+      <c r="AB4" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_epistatic_LINEAR_E1/T4Lysozyme_epistatic_predicted_vs_actual_test.png</t>
+        </is>
+      </c>
+      <c r="AC4" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_epistatic_LINEAR_E1/T4Lysozyme_epistatic_integrated_gradients_heatmap.png</t>
+        </is>
+      </c>
+      <c r="AD4" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_epistatic_LINEAR_E1/T4Lysozyme_epistatic_integrated_gradients_analysis.png</t>
+        </is>
+      </c>
+      <c r="AE4" t="inlineStr">
+        <is>
+          <t>T4 epistatic E1: anti-overfit regularized regime; dropout 0.45, lr 7.0e-4, batch 128, epochs 65, patience 17, min_epochs 12, dims 512-256-128-64.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-04-15 21:17</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>T4Lysozyme_epistatic</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>python scripts/run_integrated_gradients.py configs/synthetic/t4_tuning/T4Lysozyme_epistatic_E3_config.yaml</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>configs/synthetic/t4_tuning/T4Lysozyme_epistatic_E3_config.yaml</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_epistatic_LINEAR_E3/T4Lysozyme_epistatic_config_snapshot_20260415_194156.yaml</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_epistatic_LINEAR_E3</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_epistatic_LINEAR_E3/T4Lysozyme_epistatic_run_log_20260415_194156.txt</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>esm_attention</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>384-192-96-48</t>
+        </is>
+      </c>
+      <c r="K5" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0.0008</v>
+      </c>
+      <c r="M5" t="n">
+        <v>96</v>
+      </c>
+      <c r="N5" t="n">
+        <v>60</v>
+      </c>
+      <c r="O5" t="n">
+        <v>10</v>
+      </c>
+      <c r="P5" t="n">
+        <v>15</v>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>huber</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="S5" t="n">
+        <v>0.9539</v>
+      </c>
+      <c r="T5" t="n">
+        <v>0.0255</v>
+      </c>
+      <c r="U5" t="n">
+        <v>0.4241</v>
+      </c>
+      <c r="V5" t="n">
+        <v>0.0496</v>
+      </c>
+      <c r="W5" t="n">
+        <v>44</v>
+      </c>
+      <c r="X5" t="n">
+        <v>0.9852</v>
+      </c>
+      <c r="Y5" t="n">
+        <v>0.9928</v>
+      </c>
+      <c r="Z5" t="n">
+        <v>0.5273</v>
+      </c>
+      <c r="AA5" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_epistatic_LINEAR_E3/T4Lysozyme_epistatic_cv_loss_curves.png</t>
+        </is>
+      </c>
+      <c r="AB5" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_epistatic_LINEAR_E3/T4Lysozyme_epistatic_predicted_vs_actual_test.png</t>
+        </is>
+      </c>
+      <c r="AC5" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_epistatic_LINEAR_E3/T4Lysozyme_epistatic_integrated_gradients_heatmap.png</t>
+        </is>
+      </c>
+      <c r="AD5" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_epistatic_LINEAR_E3/T4Lysozyme_epistatic_integrated_gradients_analysis.png</t>
+        </is>
+      </c>
+      <c r="AE5" t="inlineStr">
+        <is>
+          <t>T4 epistatic E3: compact-network high-lr regime; dims 384-192-96-48, dropout 0.35, lr 8.0e-4, batch 96, epochs 60, patience 15, min_epochs 10.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2026-04-15 21:18</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>T4Lysozyme_epistatic</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>python scripts/run_integrated_gradients.py configs/synthetic/t4_tuning/T4Lysozyme_epistatic_E2_config.yaml</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>configs/synthetic/t4_tuning/T4Lysozyme_epistatic_E2_config.yaml</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_epistatic_LINEAR_E2/T4Lysozyme_epistatic_config_snapshot_20260415_194130.yaml</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_epistatic_LINEAR_E2</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_epistatic_LINEAR_E2/T4Lysozyme_epistatic_run_log_20260415_194130.txt</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>esm_attention</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>512-256-128-64</t>
+        </is>
+      </c>
+      <c r="K6" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0.00055</v>
+      </c>
+      <c r="M6" t="n">
+        <v>96</v>
+      </c>
+      <c r="N6" t="n">
+        <v>75</v>
+      </c>
+      <c r="O6" t="n">
+        <v>14</v>
+      </c>
+      <c r="P6" t="n">
+        <v>20</v>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>huber</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="S6" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="T6" t="n">
+        <v>0.0259</v>
+      </c>
+      <c r="U6" t="n">
+        <v>0.392</v>
+      </c>
+      <c r="V6" t="n">
+        <v>0.0329</v>
+      </c>
+      <c r="W6" t="n">
+        <v>57.8</v>
+      </c>
+      <c r="X6" t="n">
+        <v>0.9859</v>
+      </c>
+      <c r="Y6" t="n">
+        <v>0.993</v>
+      </c>
+      <c r="Z6" t="n">
+        <v>0.6027</v>
+      </c>
+      <c r="AA6" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_epistatic_LINEAR_E2/T4Lysozyme_epistatic_cv_loss_curves.png</t>
+        </is>
+      </c>
+      <c r="AB6" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_epistatic_LINEAR_E2/T4Lysozyme_epistatic_predicted_vs_actual_test.png</t>
+        </is>
+      </c>
+      <c r="AC6" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_epistatic_LINEAR_E2/T4Lysozyme_epistatic_integrated_gradients_heatmap.png</t>
+        </is>
+      </c>
+      <c r="AD6" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_epistatic_LINEAR_E2/T4Lysozyme_epistatic_integrated_gradients_analysis.png</t>
+        </is>
+      </c>
+      <c r="AE6" t="inlineStr">
+        <is>
+          <t>T4 epistatic E2: moderate-lr smaller-batch regime; dropout 0.40, lr 5.5e-4, batch 96, epochs 75, patience 20, min_epochs 14, dims 512-256-128-64.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F2" r:id="rId1"/>
@@ -809,7 +1317,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE2"/>
+  <dimension ref="A1:AE6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1121,6 +1629,514 @@
       <c r="AE2" t="inlineStr">
         <is>
           <t>Rana: initial run</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-04-15 16:06</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>T4Lysozyme_nonlinear</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>python scripts/run_integrated_gradients.py configs/synthetic/T4Lysozyme_nonlinear_config.yaml</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>configs/synthetic/T4Lysozyme_nonlinear_config.yaml</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_nonlinear_LINEAR/T4Lysozyme_nonlinear_config_snapshot_20260415_142055.yaml</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_nonlinear_LINEAR</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_nonlinear_LINEAR/T4Lysozyme_nonlinear_run_log_20260415_142055.txt</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>esm_attention</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>512-256-128-64</t>
+        </is>
+      </c>
+      <c r="K3" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0.0005</v>
+      </c>
+      <c r="M3" t="n">
+        <v>128</v>
+      </c>
+      <c r="N3" t="n">
+        <v>70</v>
+      </c>
+      <c r="O3" t="n">
+        <v>12</v>
+      </c>
+      <c r="P3" t="n">
+        <v>18</v>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>huber</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="S3" t="n">
+        <v>0.962</v>
+      </c>
+      <c r="T3" t="n">
+        <v>0.018</v>
+      </c>
+      <c r="U3" t="n">
+        <v>0.3999</v>
+      </c>
+      <c r="V3" t="n">
+        <v>0.0609</v>
+      </c>
+      <c r="W3" t="n">
+        <v>46.2</v>
+      </c>
+      <c r="X3" t="n">
+        <v>0.9788</v>
+      </c>
+      <c r="Y3" t="n">
+        <v>0.9893999999999999</v>
+      </c>
+      <c r="Z3" t="n">
+        <v>0.3775</v>
+      </c>
+      <c r="AA3" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_nonlinear_LINEAR/T4Lysozyme_nonlinear_cv_loss_curves.png</t>
+        </is>
+      </c>
+      <c r="AB3" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_nonlinear_LINEAR/T4Lysozyme_nonlinear_predicted_vs_actual_test.png</t>
+        </is>
+      </c>
+      <c r="AC3" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_nonlinear_LINEAR/T4Lysozyme_nonlinear_integrated_gradients_heatmap.png</t>
+        </is>
+      </c>
+      <c r="AD3" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_nonlinear_LINEAR/T4Lysozyme_nonlinear_integrated_gradients_analysis.png</t>
+        </is>
+      </c>
+      <c r="AE3" t="inlineStr">
+        <is>
+          <t>T4Lysozyme nonlinear retune from baseline: learning_rate 8e-4-&gt;5e-4, epochs 50-&gt;70, patience 15-&gt;18, min_epochs 10-&gt;12; dropout kept at 0.4 and hidden dims unchanged (512-256-128-64).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-04-15 20:07</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>T4Lysozyme_nonlinear</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>python scripts/run_integrated_gradients.py configs/synthetic/t4_tuning/T4Lysozyme_nonlinear_N1_config.yaml</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>configs/synthetic/t4_tuning/T4Lysozyme_nonlinear_N1_config.yaml</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_nonlinear_LINEAR_N1/T4Lysozyme_nonlinear_config_snapshot_20260415_194300.yaml</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_nonlinear_LINEAR_N1</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_nonlinear_LINEAR_N1/T4Lysozyme_nonlinear_run_log_20260415_194300.txt</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>esm_attention</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>512-256-128-64</t>
+        </is>
+      </c>
+      <c r="K4" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0.0008</v>
+      </c>
+      <c r="M4" t="n">
+        <v>128</v>
+      </c>
+      <c r="N4" t="n">
+        <v>55</v>
+      </c>
+      <c r="O4" t="n">
+        <v>10</v>
+      </c>
+      <c r="P4" t="n">
+        <v>15</v>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>huber</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="S4" t="n">
+        <v>0.9599</v>
+      </c>
+      <c r="T4" t="n">
+        <v>0.0298</v>
+      </c>
+      <c r="U4" t="n">
+        <v>0.3262</v>
+      </c>
+      <c r="V4" t="n">
+        <v>0.0573</v>
+      </c>
+      <c r="W4" t="n">
+        <v>44.2</v>
+      </c>
+      <c r="X4" t="n">
+        <v>0.9969</v>
+      </c>
+      <c r="Y4" t="n">
+        <v>0.9985000000000001</v>
+      </c>
+      <c r="Z4" t="n">
+        <v>0.4986</v>
+      </c>
+      <c r="AA4" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_nonlinear_LINEAR_N1/T4Lysozyme_nonlinear_cv_loss_curves.png</t>
+        </is>
+      </c>
+      <c r="AB4" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_nonlinear_LINEAR_N1/T4Lysozyme_nonlinear_predicted_vs_actual_test.png</t>
+        </is>
+      </c>
+      <c r="AC4" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_nonlinear_LINEAR_N1/T4Lysozyme_nonlinear_integrated_gradients_heatmap.png</t>
+        </is>
+      </c>
+      <c r="AD4" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_nonlinear_LINEAR_N1/T4Lysozyme_nonlinear_integrated_gradients_analysis.png</t>
+        </is>
+      </c>
+      <c r="AE4" t="inlineStr">
+        <is>
+          <t>T4 nonlinear N1: lower-dropout baseline-recovery regime; dropout 0.35, lr 8.0e-4, batch 128, epochs 55, patience 15, min_epochs 10, dims 512-256-128-64.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-04-15 20:24</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>T4Lysozyme_nonlinear</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>python scripts/run_integrated_gradients.py configs/synthetic/t4_tuning/T4Lysozyme_nonlinear_N2_config.yaml</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>configs/synthetic/t4_tuning/T4Lysozyme_nonlinear_N2_config.yaml</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_nonlinear_LINEAR_N2/T4Lysozyme_nonlinear_config_snapshot_20260415_195421.yaml</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_nonlinear_LINEAR_N2</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_nonlinear_LINEAR_N2/T4Lysozyme_nonlinear_run_log_20260415_195421.txt</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>esm_attention</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>512-256-128-64</t>
+        </is>
+      </c>
+      <c r="K5" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0.0007</v>
+      </c>
+      <c r="M5" t="n">
+        <v>128</v>
+      </c>
+      <c r="N5" t="n">
+        <v>65</v>
+      </c>
+      <c r="O5" t="n">
+        <v>12</v>
+      </c>
+      <c r="P5" t="n">
+        <v>17</v>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>huber</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="S5" t="n">
+        <v>0.9676</v>
+      </c>
+      <c r="T5" t="n">
+        <v>0.0329</v>
+      </c>
+      <c r="U5" t="n">
+        <v>0.4488</v>
+      </c>
+      <c r="V5" t="n">
+        <v>0.0684</v>
+      </c>
+      <c r="W5" t="n">
+        <v>52.8</v>
+      </c>
+      <c r="X5" t="n">
+        <v>0.9708</v>
+      </c>
+      <c r="Y5" t="n">
+        <v>0.9855</v>
+      </c>
+      <c r="Z5" t="n">
+        <v>0.4703</v>
+      </c>
+      <c r="AA5" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_nonlinear_LINEAR_N2/T4Lysozyme_nonlinear_cv_loss_curves.png</t>
+        </is>
+      </c>
+      <c r="AB5" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_nonlinear_LINEAR_N2/T4Lysozyme_nonlinear_predicted_vs_actual_test.png</t>
+        </is>
+      </c>
+      <c r="AC5" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_nonlinear_LINEAR_N2/T4Lysozyme_nonlinear_integrated_gradients_heatmap.png</t>
+        </is>
+      </c>
+      <c r="AD5" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_nonlinear_LINEAR_N2/T4Lysozyme_nonlinear_integrated_gradients_analysis.png</t>
+        </is>
+      </c>
+      <c r="AE5" t="inlineStr">
+        <is>
+          <t>T4 nonlinear N2: stronger-regularization regime; dropout 0.45, lr 7.0e-4, batch 128, epochs 65, patience 17, min_epochs 12, dims 512-256-128-64.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2026-04-15 21:42</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>T4Lysozyme_nonlinear</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>python scripts/run_integrated_gradients.py configs/synthetic/t4_tuning/T4Lysozyme_nonlinear_N3_config.yaml</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>configs/synthetic/t4_tuning/T4Lysozyme_nonlinear_N3_config.yaml</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_nonlinear_LINEAR_N3/T4Lysozyme_nonlinear_config_snapshot_20260415_200110.yaml</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_nonlinear_LINEAR_N3</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_nonlinear_LINEAR_N3/T4Lysozyme_nonlinear_run_log_20260415_200110.txt</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>esm_attention</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>384-192-96-48</t>
+        </is>
+      </c>
+      <c r="K6" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0.0009</v>
+      </c>
+      <c r="M6" t="n">
+        <v>96</v>
+      </c>
+      <c r="N6" t="n">
+        <v>55</v>
+      </c>
+      <c r="O6" t="n">
+        <v>10</v>
+      </c>
+      <c r="P6" t="n">
+        <v>14</v>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>huber</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="S6" t="n">
+        <v>0.9552</v>
+      </c>
+      <c r="T6" t="n">
+        <v>0.0191</v>
+      </c>
+      <c r="U6" t="n">
+        <v>0.3882</v>
+      </c>
+      <c r="V6" t="n">
+        <v>0.07829999999999999</v>
+      </c>
+      <c r="W6" t="n">
+        <v>41.6</v>
+      </c>
+      <c r="X6" t="n">
+        <v>0.9976</v>
+      </c>
+      <c r="Y6" t="n">
+        <v>0.9989</v>
+      </c>
+      <c r="Z6" t="n">
+        <v>0.5651</v>
+      </c>
+      <c r="AA6" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_nonlinear_LINEAR_N3/T4Lysozyme_nonlinear_cv_loss_curves.png</t>
+        </is>
+      </c>
+      <c r="AB6" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_nonlinear_LINEAR_N3/T4Lysozyme_nonlinear_predicted_vs_actual_test.png</t>
+        </is>
+      </c>
+      <c r="AC6" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_nonlinear_LINEAR_N3/T4Lysozyme_nonlinear_integrated_gradients_heatmap.png</t>
+        </is>
+      </c>
+      <c r="AD6" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_nonlinear_LINEAR_N3/T4Lysozyme_nonlinear_integrated_gradients_analysis.png</t>
+        </is>
+      </c>
+      <c r="AE6" t="inlineStr">
+        <is>
+          <t>T4 nonlinear N3: compact-network rank-focused regime; dims 384-192-96-48, dropout 0.40, lr 9.0e-4, batch 96, epochs 55, patience 14, min_epochs 10.</t>
         </is>
       </c>
     </row>
@@ -5104,7 +6120,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE2"/>
+  <dimension ref="A1:AE6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -5419,6 +6435,514 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-04-15 12:46</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>T4Lysozyme_additive</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>python scripts/run_integrated_gradients.py configs/synthetic/T4Lysozyme_additive_config.yaml</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>configs/synthetic/T4Lysozyme_additive_config.yaml</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_additive_LINEAR/T4Lysozyme_additive_config_snapshot_20260415_105021.yaml</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_additive_LINEAR</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_additive_LINEAR/T4Lysozyme_additive_run_log_20260415_105021.txt</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>esm_attention</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>512-256-128-64</t>
+        </is>
+      </c>
+      <c r="K3" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0.0005999999999999999</v>
+      </c>
+      <c r="M3" t="n">
+        <v>128</v>
+      </c>
+      <c r="N3" t="n">
+        <v>80</v>
+      </c>
+      <c r="O3" t="n">
+        <v>15</v>
+      </c>
+      <c r="P3" t="n">
+        <v>20</v>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>huber</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="S3" t="n">
+        <v>0.9324</v>
+      </c>
+      <c r="T3" t="n">
+        <v>0.039</v>
+      </c>
+      <c r="U3" t="n">
+        <v>0.4401</v>
+      </c>
+      <c r="V3" t="n">
+        <v>0.073</v>
+      </c>
+      <c r="W3" t="n">
+        <v>65.59999999999999</v>
+      </c>
+      <c r="X3" t="n">
+        <v>0.9522</v>
+      </c>
+      <c r="Y3" t="n">
+        <v>0.976</v>
+      </c>
+      <c r="Z3" t="n">
+        <v>0.4474</v>
+      </c>
+      <c r="AA3" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_additive_LINEAR/T4Lysozyme_additive_cv_loss_curves.png</t>
+        </is>
+      </c>
+      <c r="AB3" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_additive_LINEAR/T4Lysozyme_additive_predicted_vs_actual_test.png</t>
+        </is>
+      </c>
+      <c r="AC3" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_additive_LINEAR/T4Lysozyme_additive_integrated_gradients_heatmap.png</t>
+        </is>
+      </c>
+      <c r="AD3" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_additive_LINEAR/T4Lysozyme_additive_integrated_gradients_analysis.png</t>
+        </is>
+      </c>
+      <c r="AE3" t="inlineStr">
+        <is>
+          <t>T4Lysozyme additive retune from baseline: dropout 0.4-&gt;0.35, learning_rate 8e-4-&gt;6e-4, epochs 50-&gt;80, patience 15-&gt;20, min_epochs 10-&gt;15; hidden dims unchanged.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-04-15 21:28</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>T4Lysozyme_additive</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>python scripts/run_integrated_gradients.py configs/synthetic/t4_tuning/T4Lysozyme_additive_A2_config.yaml</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>configs/synthetic/t4_tuning/T4Lysozyme_additive_A2_config.yaml</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_additive_LINEAR_A2/T4Lysozyme_additive_config_snapshot_20260415_204443.yaml</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_additive_LINEAR_A2</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_additive_LINEAR_A2/T4Lysozyme_additive_run_log_20260415_204443.txt</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>esm_attention</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>512-256-128-64</t>
+        </is>
+      </c>
+      <c r="K4" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0.00055</v>
+      </c>
+      <c r="M4" t="n">
+        <v>128</v>
+      </c>
+      <c r="N4" t="n">
+        <v>90</v>
+      </c>
+      <c r="O4" t="n">
+        <v>16</v>
+      </c>
+      <c r="P4" t="n">
+        <v>22</v>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>huber</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="S4" t="n">
+        <v>0.9417</v>
+      </c>
+      <c r="T4" t="n">
+        <v>0.0268</v>
+      </c>
+      <c r="U4" t="n">
+        <v>0.413</v>
+      </c>
+      <c r="V4" t="n">
+        <v>0.0483</v>
+      </c>
+      <c r="W4" t="n">
+        <v>72.59999999999999</v>
+      </c>
+      <c r="X4" t="n">
+        <v>0.9716</v>
+      </c>
+      <c r="Y4" t="n">
+        <v>0.9859</v>
+      </c>
+      <c r="Z4" t="n">
+        <v>0.4536</v>
+      </c>
+      <c r="AA4" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_additive_LINEAR_A2/T4Lysozyme_additive_cv_loss_curves.png</t>
+        </is>
+      </c>
+      <c r="AB4" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_additive_LINEAR_A2/T4Lysozyme_additive_predicted_vs_actual_test.png</t>
+        </is>
+      </c>
+      <c r="AC4" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_additive_LINEAR_A2/T4Lysozyme_additive_integrated_gradients_heatmap.png</t>
+        </is>
+      </c>
+      <c r="AD4" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_additive_LINEAR_A2/T4Lysozyme_additive_integrated_gradients_analysis.png</t>
+        </is>
+      </c>
+      <c r="AE4" t="inlineStr">
+        <is>
+          <t>Retry after initial failed batch due environment race; additive A2.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-04-15 21:28</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>T4Lysozyme_additive</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>python scripts/run_integrated_gradients.py configs/synthetic/t4_tuning/T4Lysozyme_additive_A1_config.yaml</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>configs/synthetic/t4_tuning/T4Lysozyme_additive_A1_config.yaml</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_additive_LINEAR_A1/T4Lysozyme_additive_config_snapshot_20260415_194017.yaml</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_additive_LINEAR_A1</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_additive_LINEAR_A1/T4Lysozyme_additive_run_log_20260415_194017.txt</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>esm_attention</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>512-256-128-64</t>
+        </is>
+      </c>
+      <c r="K5" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0.00045</v>
+      </c>
+      <c r="M5" t="n">
+        <v>96</v>
+      </c>
+      <c r="N5" t="n">
+        <v>110</v>
+      </c>
+      <c r="O5" t="n">
+        <v>20</v>
+      </c>
+      <c r="P5" t="n">
+        <v>26</v>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>huber</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="S5" t="n">
+        <v>0.9363</v>
+      </c>
+      <c r="T5" t="n">
+        <v>0.0291</v>
+      </c>
+      <c r="U5" t="n">
+        <v>0.4784</v>
+      </c>
+      <c r="V5" t="n">
+        <v>0.0563</v>
+      </c>
+      <c r="W5" t="n">
+        <v>85.59999999999999</v>
+      </c>
+      <c r="X5" t="n">
+        <v>0.9839</v>
+      </c>
+      <c r="Y5" t="n">
+        <v>0.992</v>
+      </c>
+      <c r="Z5" t="n">
+        <v>0.5508</v>
+      </c>
+      <c r="AA5" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_additive_LINEAR_A1/T4Lysozyme_additive_cv_loss_curves.png</t>
+        </is>
+      </c>
+      <c r="AB5" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_additive_LINEAR_A1/T4Lysozyme_additive_predicted_vs_actual_test.png</t>
+        </is>
+      </c>
+      <c r="AC5" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_additive_LINEAR_A1/T4Lysozyme_additive_integrated_gradients_heatmap.png</t>
+        </is>
+      </c>
+      <c r="AD5" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_additive_LINEAR_A1/T4Lysozyme_additive_integrated_gradients_analysis.png</t>
+        </is>
+      </c>
+      <c r="AE5" t="inlineStr">
+        <is>
+          <t>T4 additive A1: low-dropout long-train regime; lr 4.5e-4, batch 96, epochs 110, patience 26, min_epochs 20, dims 512-256-128-64.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2026-04-15 21:30</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>T4Lysozyme_additive</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>python scripts/run_integrated_gradients.py configs/synthetic/t4_tuning/T4Lysozyme_additive_A3_config.yaml</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>configs/synthetic/t4_tuning/T4Lysozyme_additive_A3_config.yaml</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_additive_LINEAR_A3/T4Lysozyme_additive_config_snapshot_20260415_194013.yaml</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_additive_LINEAR_A3</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_additive_LINEAR_A3/T4Lysozyme_additive_run_log_20260415_194013.txt</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>esm_attention</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>384-192-96-48</t>
+        </is>
+      </c>
+      <c r="K6" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0.00075</v>
+      </c>
+      <c r="M6" t="n">
+        <v>96</v>
+      </c>
+      <c r="N6" t="n">
+        <v>70</v>
+      </c>
+      <c r="O6" t="n">
+        <v>12</v>
+      </c>
+      <c r="P6" t="n">
+        <v>18</v>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>huber</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="S6" t="n">
+        <v>0.9497</v>
+      </c>
+      <c r="T6" t="n">
+        <v>0.038</v>
+      </c>
+      <c r="U6" t="n">
+        <v>0.5052</v>
+      </c>
+      <c r="V6" t="n">
+        <v>0.0308</v>
+      </c>
+      <c r="W6" t="n">
+        <v>55.8</v>
+      </c>
+      <c r="X6" t="n">
+        <v>0.9765</v>
+      </c>
+      <c r="Y6" t="n">
+        <v>0.9885</v>
+      </c>
+      <c r="Z6" t="n">
+        <v>0.4504</v>
+      </c>
+      <c r="AA6" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_additive_LINEAR_A3/T4Lysozyme_additive_cv_loss_curves.png</t>
+        </is>
+      </c>
+      <c r="AB6" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_additive_LINEAR_A3/T4Lysozyme_additive_predicted_vs_actual_test.png</t>
+        </is>
+      </c>
+      <c r="AC6" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_additive_LINEAR_A3/T4Lysozyme_additive_integrated_gradients_heatmap.png</t>
+        </is>
+      </c>
+      <c r="AD6" t="inlineStr">
+        <is>
+          <t>results/synthetic/T4Lysozyme_additive_LINEAR_A3/T4Lysozyme_additive_integrated_gradients_analysis.png</t>
+        </is>
+      </c>
+      <c r="AE6" t="inlineStr">
+        <is>
+          <t>T4 additive A3: compact-network faster regime; dims 384-192-96-48, dropout 0.35, lr 7.5e-4, batch 96, epochs 70, patience 18, min_epochs 12.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F2" r:id="rId1"/>

</xml_diff>

<commit_message>
synth GB1  LINEAR results
</commit_message>
<xml_diff>
--- a/experiment_tracker.xlsx
+++ b/experiment_tracker.xlsx
@@ -1021,7 +1021,6 @@
           <t>python scripts/run_integrated_gradients.py configs/synthetic/T4Lysozyme_nonlinear_config.yaml</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
       <c r="F2" s="3" t="inlineStr">
         <is>
           <t>results/synthetic/T4Lysozyme_nonlinear_LINEAR/T4Lysozyme_nonlinear_config_snapshot_20260414_201415.yaml</t>
@@ -2015,7 +2014,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -2070,18 +2069,18 @@
           <t>GB1_additive</t>
         </is>
       </c>
-      <c r="B2" s="2" t="n">
-        <v>-0.0425</v>
-      </c>
-      <c r="C2" s="2" t="n">
-        <v>-0.06560000000000001</v>
+      <c r="B2" s="4" t="n">
+        <v>0.8463000000000001</v>
+      </c>
+      <c r="C2" s="4" t="n">
+        <v>0.9134</v>
       </c>
       <c r="D2" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-04-10 18:24</t>
+          <t>2026-04-17 13:34</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -2263,6 +2262,58 @@
       <c r="F9" t="inlineStr">
         <is>
           <t>results/synthetic/T4Lysozyme_nonlinear_LINEAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>GB1_epistatic</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="n">
+        <v>0.8379</v>
+      </c>
+      <c r="C10" s="4" t="n">
+        <v>0.8935</v>
+      </c>
+      <c r="D10" t="n">
+        <v>5</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>2026-04-17 13:36</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_epistatic_LINEAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>GB1_nonlinear</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="n">
+        <v>0.8115</v>
+      </c>
+      <c r="C11" s="4" t="n">
+        <v>0.8848</v>
+      </c>
+      <c r="D11" t="n">
+        <v>5</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>2026-04-17 13:58</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_nonlinear_LINEAR</t>
         </is>
       </c>
     </row>
@@ -2277,7 +2328,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE3"/>
+  <dimension ref="A1:AE11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -2724,6 +2775,982 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-04-16 11:59</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>GB1_additive</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>python scripts/run_integrated_gradients.py configs/synthetic/GB1_additive_config.yaml</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_additive_LINEAR/GB1_additive_config_snapshot_20260415_145841.yaml</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_additive_LINEAR</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_additive_LINEAR/GB1_additive_run_log_20260415_145840.txt</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>esm_attention</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>256-128-64-32</t>
+        </is>
+      </c>
+      <c r="K4" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="M4" t="n">
+        <v>64</v>
+      </c>
+      <c r="N4" t="n">
+        <v>50</v>
+      </c>
+      <c r="O4" t="n">
+        <v>10</v>
+      </c>
+      <c r="P4" t="n">
+        <v>15</v>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>huber</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="S4" s="4" t="n">
+        <v>0.7449</v>
+      </c>
+      <c r="T4" t="n">
+        <v>0.022</v>
+      </c>
+      <c r="U4" s="4" t="n">
+        <v>0.8656</v>
+      </c>
+      <c r="V4" t="n">
+        <v>0.0074</v>
+      </c>
+      <c r="W4" t="n">
+        <v>45.4</v>
+      </c>
+      <c r="X4" s="4" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="Y4" s="4" t="n">
+        <v>0.9117</v>
+      </c>
+      <c r="Z4" s="4" t="n">
+        <v>0.8874</v>
+      </c>
+      <c r="AA4" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_additive_LINEAR/GB1_additive_cv_loss_curves.png</t>
+        </is>
+      </c>
+      <c r="AB4" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_additive_LINEAR/GB1_additive_predicted_vs_actual_test.png</t>
+        </is>
+      </c>
+      <c r="AC4" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_additive_LINEAR/GB1_additive_integrated_gradients_heatmap.png</t>
+        </is>
+      </c>
+      <c r="AD4" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_additive_LINEAR/GB1_additive_integrated_gradients_analysis.png</t>
+        </is>
+      </c>
+      <c r="AE4" t="inlineStr">
+        <is>
+          <t>Will: initial run</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-04-16 12:20</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>GB1_additive</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>python scripts/run_integrated_gradients.py configs/synthetic/GB1_additive_config.yaml</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_additive_LINEAR/GB1_additive_config_snapshot_20260415_145841.yaml</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_additive_LINEAR</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_additive_LINEAR/GB1_additive_run_log_20260415_145840.txt</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>esm_attention</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>256-128-64-32</t>
+        </is>
+      </c>
+      <c r="K5" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="M5" t="n">
+        <v>64</v>
+      </c>
+      <c r="N5" t="n">
+        <v>50</v>
+      </c>
+      <c r="O5" t="n">
+        <v>10</v>
+      </c>
+      <c r="P5" t="n">
+        <v>15</v>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>huber</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="S5" s="4" t="n">
+        <v>0.7449</v>
+      </c>
+      <c r="T5" t="n">
+        <v>0.022</v>
+      </c>
+      <c r="U5" s="4" t="n">
+        <v>0.8656</v>
+      </c>
+      <c r="V5" t="n">
+        <v>0.0074</v>
+      </c>
+      <c r="W5" t="n">
+        <v>45.4</v>
+      </c>
+      <c r="X5" s="4" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="Y5" s="4" t="n">
+        <v>0.9117</v>
+      </c>
+      <c r="Z5" s="4" t="n">
+        <v>0.8874</v>
+      </c>
+      <c r="AA5" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_additive_LINEAR/GB1_additive_cv_loss_curves.png</t>
+        </is>
+      </c>
+      <c r="AB5" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_additive_LINEAR/GB1_additive_predicted_vs_actual_test.png</t>
+        </is>
+      </c>
+      <c r="AC5" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_additive_LINEAR/GB1_additive_integrated_gradients_heatmap.png</t>
+        </is>
+      </c>
+      <c r="AD5" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_additive_LINEAR/GB1_additive_integrated_gradients_analysis.png</t>
+        </is>
+      </c>
+      <c r="AE5" t="inlineStr">
+        <is>
+          <t>Will: initial run</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2026-04-16 12:36</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>GB1_additive</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>python scripts/run_integrated_gradients.py configs/synthetic/GB1_additive_config.yaml</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_additive_LINEAR/GB1_additive_config_snapshot_20260416_122524.yaml</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_additive_LINEAR</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_additive_LINEAR/GB1_additive_run_log_20260416_122524.txt</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>esm_attention</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>512-256-128-64</t>
+        </is>
+      </c>
+      <c r="K6" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="M6" t="n">
+        <v>64</v>
+      </c>
+      <c r="N6" t="n">
+        <v>50</v>
+      </c>
+      <c r="O6" t="n">
+        <v>10</v>
+      </c>
+      <c r="P6" t="n">
+        <v>15</v>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>huber</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="S6" s="4" t="n">
+        <v>0.7717000000000001</v>
+      </c>
+      <c r="T6" t="n">
+        <v>0.0302</v>
+      </c>
+      <c r="U6" s="4" t="n">
+        <v>0.8875</v>
+      </c>
+      <c r="V6" t="n">
+        <v>0.0117</v>
+      </c>
+      <c r="W6" t="n">
+        <v>47.2</v>
+      </c>
+      <c r="X6" s="4" t="n">
+        <v>0.842</v>
+      </c>
+      <c r="Y6" s="4" t="n">
+        <v>0.9177</v>
+      </c>
+      <c r="Z6" s="4" t="n">
+        <v>0.8997000000000001</v>
+      </c>
+      <c r="AA6" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_additive_LINEAR/GB1_additive_cv_loss_curves.png</t>
+        </is>
+      </c>
+      <c r="AB6" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_additive_LINEAR/GB1_additive_predicted_vs_actual_test.png</t>
+        </is>
+      </c>
+      <c r="AC6" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_additive_LINEAR/GB1_additive_integrated_gradients_heatmap.png</t>
+        </is>
+      </c>
+      <c r="AD6" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_additive_LINEAR/GB1_additive_integrated_gradients_analysis.png</t>
+        </is>
+      </c>
+      <c r="AE6" t="inlineStr">
+        <is>
+          <t>Will: doubled hidden dimensions</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2026-04-17 13:34</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>GB1_additive</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>python scripts/run_integrated_gradients.py configs/synthetic/GB1_additive_config.yaml</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_additive_LINEAR/GB1_additive_config_snapshot_20260417_132916.yaml</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_additive_LINEAR</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_additive_LINEAR/GB1_additive_run_log_20260417_132915.txt</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>esm_attention</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>512-256-128-64</t>
+        </is>
+      </c>
+      <c r="K7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="L7" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="M7" t="n">
+        <v>64</v>
+      </c>
+      <c r="N7" t="n">
+        <v>50</v>
+      </c>
+      <c r="O7" t="n">
+        <v>10</v>
+      </c>
+      <c r="P7" t="n">
+        <v>15</v>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>huber</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="S7" s="4" t="n">
+        <v>0.6127</v>
+      </c>
+      <c r="T7" t="n">
+        <v>0.0822</v>
+      </c>
+      <c r="U7" s="4" t="n">
+        <v>0.8051</v>
+      </c>
+      <c r="V7" t="n">
+        <v>0.0466</v>
+      </c>
+      <c r="W7" t="n">
+        <v>45</v>
+      </c>
+      <c r="X7" s="4" t="n">
+        <v>0.8463000000000001</v>
+      </c>
+      <c r="Y7" s="4" t="n">
+        <v>0.9225</v>
+      </c>
+      <c r="Z7" s="4" t="n">
+        <v>0.9134</v>
+      </c>
+      <c r="AA7" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_additive_LINEAR/GB1_additive_cv_loss_curves.png</t>
+        </is>
+      </c>
+      <c r="AB7" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_additive_LINEAR/GB1_additive_predicted_vs_actual_test.png</t>
+        </is>
+      </c>
+      <c r="AC7" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_additive_LINEAR/GB1_additive_integrated_gradients_heatmap.png</t>
+        </is>
+      </c>
+      <c r="AD7" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_additive_LINEAR/GB1_additive_integrated_gradients_analysis.png</t>
+        </is>
+      </c>
+      <c r="AE7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Will:Higer LR &amp; DrpOut </t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2026-04-17 13:39</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>GB1_additive</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>python scripts/run_integrated_gradients.py configs/synthetic/GB1_additive_config.yaml</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_additive_LINEAR/GB1_additive_config_snapshot_20260417_133447.yaml</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_additive_LINEAR</t>
+        </is>
+      </c>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_additive_LINEAR/GB1_additive_run_log_20260417_133447.txt</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>esm_attention</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>512-256-128-64</t>
+        </is>
+      </c>
+      <c r="K8" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="L8" t="n">
+        <v>0.0005</v>
+      </c>
+      <c r="M8" t="n">
+        <v>64</v>
+      </c>
+      <c r="N8" t="n">
+        <v>50</v>
+      </c>
+      <c r="O8" t="n">
+        <v>10</v>
+      </c>
+      <c r="P8" t="n">
+        <v>15</v>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>huber</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="S8" s="4" t="n">
+        <v>0.7517</v>
+      </c>
+      <c r="T8" t="n">
+        <v>0.0222</v>
+      </c>
+      <c r="U8" s="4" t="n">
+        <v>0.8774999999999999</v>
+      </c>
+      <c r="V8" t="n">
+        <v>0.0077</v>
+      </c>
+      <c r="W8" t="n">
+        <v>46.4</v>
+      </c>
+      <c r="X8" s="4" t="n">
+        <v>0.8178</v>
+      </c>
+      <c r="Y8" s="4" t="n">
+        <v>0.9049</v>
+      </c>
+      <c r="Z8" s="4" t="n">
+        <v>0.8802</v>
+      </c>
+      <c r="AA8" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_additive_LINEAR/GB1_additive_cv_loss_curves.png</t>
+        </is>
+      </c>
+      <c r="AB8" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_additive_LINEAR/GB1_additive_predicted_vs_actual_test.png</t>
+        </is>
+      </c>
+      <c r="AC8" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_additive_LINEAR/GB1_additive_integrated_gradients_heatmap.png</t>
+        </is>
+      </c>
+      <c r="AD8" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_additive_LINEAR/GB1_additive_integrated_gradients_analysis.png</t>
+        </is>
+      </c>
+      <c r="AE8" t="inlineStr">
+        <is>
+          <t>Will: Lower LR and DrpOut</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2026-04-17 13:47</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>GB1_additive</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>python scripts/run_integrated_gradients.py configs/synthetic/GB1_additive_config.yaml</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_additive_LINEAR/GB1_additive_config_snapshot_20260417_134320.yaml</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_additive_LINEAR</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_additive_LINEAR/GB1_additive_run_log_20260417_134319.txt</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>esm_attention</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>128-64-32-16</t>
+        </is>
+      </c>
+      <c r="K9" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="L9" t="n">
+        <v>0.0005</v>
+      </c>
+      <c r="M9" t="n">
+        <v>64</v>
+      </c>
+      <c r="N9" t="n">
+        <v>50</v>
+      </c>
+      <c r="O9" t="n">
+        <v>10</v>
+      </c>
+      <c r="P9" t="n">
+        <v>15</v>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>huber</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="S9" s="4" t="n">
+        <v>0.7143</v>
+      </c>
+      <c r="T9" t="n">
+        <v>0.0258</v>
+      </c>
+      <c r="U9" s="4" t="n">
+        <v>0.8561</v>
+      </c>
+      <c r="V9" t="n">
+        <v>0.008999999999999999</v>
+      </c>
+      <c r="W9" t="n">
+        <v>47.4</v>
+      </c>
+      <c r="X9" s="4" t="n">
+        <v>0.8067</v>
+      </c>
+      <c r="Y9" s="4" t="n">
+        <v>0.8986</v>
+      </c>
+      <c r="Z9" s="4" t="n">
+        <v>0.8751</v>
+      </c>
+      <c r="AA9" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_additive_LINEAR/GB1_additive_cv_loss_curves.png</t>
+        </is>
+      </c>
+      <c r="AB9" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_additive_LINEAR/GB1_additive_predicted_vs_actual_test.png</t>
+        </is>
+      </c>
+      <c r="AC9" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_additive_LINEAR/GB1_additive_integrated_gradients_heatmap.png</t>
+        </is>
+      </c>
+      <c r="AD9" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_additive_LINEAR/GB1_additive_integrated_gradients_analysis.png</t>
+        </is>
+      </c>
+      <c r="AE9" t="inlineStr">
+        <is>
+          <t>Will: half initial hidden dims</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2026-04-17 13:50</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>GB1_additive</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>python scripts/run_integrated_gradients.py configs/synthetic/GB1_additive_config.yaml</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_additive_LINEAR/GB1_additive_config_snapshot_20260417_134830.yaml</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_additive_LINEAR</t>
+        </is>
+      </c>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_additive_LINEAR/GB1_additive_run_log_20260417_134829.txt</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>esm_attention</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>128-64-32-16</t>
+        </is>
+      </c>
+      <c r="K10" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="L10" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="M10" t="n">
+        <v>64</v>
+      </c>
+      <c r="N10" t="n">
+        <v>50</v>
+      </c>
+      <c r="O10" t="n">
+        <v>10</v>
+      </c>
+      <c r="P10" t="n">
+        <v>15</v>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>huber</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="S10" s="4" t="n">
+        <v>0.7143</v>
+      </c>
+      <c r="T10" t="n">
+        <v>0.0258</v>
+      </c>
+      <c r="U10" s="4" t="n">
+        <v>0.8561</v>
+      </c>
+      <c r="V10" t="n">
+        <v>0.008999999999999999</v>
+      </c>
+      <c r="W10" t="n">
+        <v>47.4</v>
+      </c>
+      <c r="X10" s="4" t="n">
+        <v>0.8067</v>
+      </c>
+      <c r="Y10" s="4" t="n">
+        <v>0.8986</v>
+      </c>
+      <c r="Z10" s="4" t="n">
+        <v>0.8751</v>
+      </c>
+      <c r="AA10" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_additive_LINEAR/GB1_additive_cv_loss_curves.png</t>
+        </is>
+      </c>
+      <c r="AB10" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_additive_LINEAR/GB1_additive_predicted_vs_actual_test.png</t>
+        </is>
+      </c>
+      <c r="AC10" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_additive_LINEAR/GB1_additive_integrated_gradients_heatmap.png</t>
+        </is>
+      </c>
+      <c r="AD10" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_additive_LINEAR/GB1_additive_integrated_gradients_analysis.png</t>
+        </is>
+      </c>
+      <c r="AE10" t="inlineStr">
+        <is>
+          <t>Will: higher LR and DrpOut</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2026-04-17 13:53</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>GB1_additive</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>python scripts/run_integrated_gradients.py configs/synthetic/GB1_additive_config.yaml</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_additive_LINEAR/GB1_additive_config_snapshot_20260417_134830.yaml</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_additive_LINEAR</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_additive_LINEAR/GB1_additive_run_log_20260417_134829.txt</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>esm_attention</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>128-64-32-16</t>
+        </is>
+      </c>
+      <c r="K11" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="L11" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="M11" t="n">
+        <v>64</v>
+      </c>
+      <c r="N11" t="n">
+        <v>50</v>
+      </c>
+      <c r="O11" t="n">
+        <v>10</v>
+      </c>
+      <c r="P11" t="n">
+        <v>15</v>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>huber</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="S11" s="4" t="n">
+        <v>0.7615</v>
+      </c>
+      <c r="T11" t="n">
+        <v>0.0135</v>
+      </c>
+      <c r="U11" s="4" t="n">
+        <v>0.8819</v>
+      </c>
+      <c r="V11" t="n">
+        <v>0.0102</v>
+      </c>
+      <c r="W11" t="n">
+        <v>47.4</v>
+      </c>
+      <c r="X11" s="4" t="n">
+        <v>0.8137</v>
+      </c>
+      <c r="Y11" s="4" t="n">
+        <v>0.905</v>
+      </c>
+      <c r="Z11" s="4" t="n">
+        <v>0.8871</v>
+      </c>
+      <c r="AA11" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_additive_LINEAR/GB1_additive_cv_loss_curves.png</t>
+        </is>
+      </c>
+      <c r="AB11" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_additive_LINEAR/GB1_additive_predicted_vs_actual_test.png</t>
+        </is>
+      </c>
+      <c r="AC11" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_additive_LINEAR/GB1_additive_integrated_gradients_heatmap.png</t>
+        </is>
+      </c>
+      <c r="AD11" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_additive_LINEAR/GB1_additive_integrated_gradients_analysis.png</t>
+        </is>
+      </c>
+      <c r="AE11" t="inlineStr">
+        <is>
+          <t>Will: normal LR and DrpOut</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F2" r:id="rId1"/>
@@ -2738,6 +3765,54 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB3" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC3" r:id="rId11"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD3" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F4" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H4" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA4" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB4" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC4" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD4" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F5" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H5" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA5" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB5" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC5" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD5" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F6" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA6" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB6" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC6" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD6" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F7" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H7" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA7" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB7" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC7" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD7" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H8" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA8" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB8" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC8" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD8" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F9" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H9" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA9" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB9" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC9" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD9" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F10" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H10" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA10" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB10" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC10" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD10" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F11" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H11" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA11" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB11" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC11" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD11" r:id="rId60"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2749,7 +3824,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE1"/>
+  <dimension ref="A1:AE6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -2942,7 +4017,650 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2026-04-17 13:17</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>GB1_epistatic</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>python scripts/run_integrated_gradients.py configs/synthetic/GB1_epistatic_config.yaml</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_epistatic_LINEAR/GB1_epistatic_config_snapshot_20260416_123720.yaml</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_epistatic_LINEAR</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_epistatic_LINEAR/GB1_epistatic_run_log_20260416_123720.txt</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>esm_attention</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>256-128-64-32</t>
+        </is>
+      </c>
+      <c r="K2" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="M2" t="n">
+        <v>64</v>
+      </c>
+      <c r="N2" t="n">
+        <v>50</v>
+      </c>
+      <c r="O2" t="n">
+        <v>10</v>
+      </c>
+      <c r="P2" t="n">
+        <v>15</v>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>huber</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="S2" s="4" t="n">
+        <v>0.7529</v>
+      </c>
+      <c r="T2" t="n">
+        <v>0.0277</v>
+      </c>
+      <c r="U2" s="4" t="n">
+        <v>0.8811</v>
+      </c>
+      <c r="V2" t="n">
+        <v>0.0124</v>
+      </c>
+      <c r="W2" t="n">
+        <v>44.2</v>
+      </c>
+      <c r="X2" s="4" t="n">
+        <v>0.8237</v>
+      </c>
+      <c r="Y2" s="4" t="n">
+        <v>0.9079</v>
+      </c>
+      <c r="Z2" s="4" t="n">
+        <v>0.8924</v>
+      </c>
+      <c r="AA2" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_epistatic_LINEAR/GB1_epistatic_cv_loss_curves.png</t>
+        </is>
+      </c>
+      <c r="AB2" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_epistatic_LINEAR/GB1_epistatic_predicted_vs_actual_test.png</t>
+        </is>
+      </c>
+      <c r="AC2" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_epistatic_LINEAR/GB1_epistatic_integrated_gradients_heatmap.png</t>
+        </is>
+      </c>
+      <c r="AD2" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_epistatic_LINEAR/GB1_epistatic_integrated_gradients_analysis.png</t>
+        </is>
+      </c>
+      <c r="AE2" t="inlineStr">
+        <is>
+          <t>Will: initial run</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-04-17 13:36</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>GB1_epistatic</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>python scripts/run_integrated_gradients.py configs/synthetic/GB1_epistatic_config.yaml</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_epistatic_LINEAR/GB1_epistatic_config_snapshot_20260417_133023.yaml</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_epistatic_LINEAR</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_epistatic_LINEAR/GB1_epistatic_run_log_20260417_133023.txt</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>esm_attention</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>512-256-128-64</t>
+        </is>
+      </c>
+      <c r="K3" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="M3" t="n">
+        <v>64</v>
+      </c>
+      <c r="N3" t="n">
+        <v>50</v>
+      </c>
+      <c r="O3" t="n">
+        <v>10</v>
+      </c>
+      <c r="P3" t="n">
+        <v>15</v>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>huber</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="S3" s="4" t="n">
+        <v>0.7327</v>
+      </c>
+      <c r="T3" t="n">
+        <v>0.052</v>
+      </c>
+      <c r="U3" s="4" t="n">
+        <v>0.8614000000000001</v>
+      </c>
+      <c r="V3" t="n">
+        <v>0.0201</v>
+      </c>
+      <c r="W3" t="n">
+        <v>47.4</v>
+      </c>
+      <c r="X3" s="4" t="n">
+        <v>0.8379</v>
+      </c>
+      <c r="Y3" s="4" t="n">
+        <v>0.9155</v>
+      </c>
+      <c r="Z3" s="4" t="n">
+        <v>0.8935</v>
+      </c>
+      <c r="AA3" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_epistatic_LINEAR/GB1_epistatic_cv_loss_curves.png</t>
+        </is>
+      </c>
+      <c r="AB3" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_epistatic_LINEAR/GB1_epistatic_predicted_vs_actual_test.png</t>
+        </is>
+      </c>
+      <c r="AC3" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_epistatic_LINEAR/GB1_epistatic_integrated_gradients_heatmap.png</t>
+        </is>
+      </c>
+      <c r="AD3" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_epistatic_LINEAR/GB1_epistatic_integrated_gradients_analysis.png</t>
+        </is>
+      </c>
+      <c r="AE3" t="inlineStr">
+        <is>
+          <t>Will: Double hidden dims</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-04-17 13:51</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>GB1_epistatic</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>python scripts/run_integrated_gradients.py configs/synthetic/GB1_epistatic_config.yaml</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_epistatic_LINEAR/GB1_epistatic_config_snapshot_20260417_134425.yaml</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_epistatic_LINEAR</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_epistatic_LINEAR/GB1_epistatic_run_log_20260417_134425.txt</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>esm_attention</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>512-256-128-64</t>
+        </is>
+      </c>
+      <c r="K4" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="M4" t="n">
+        <v>64</v>
+      </c>
+      <c r="N4" t="n">
+        <v>50</v>
+      </c>
+      <c r="O4" t="n">
+        <v>10</v>
+      </c>
+      <c r="P4" t="n">
+        <v>15</v>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>huber</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="S4" s="4" t="n">
+        <v>0.6672</v>
+      </c>
+      <c r="T4" t="n">
+        <v>0.0606</v>
+      </c>
+      <c r="U4" s="4" t="n">
+        <v>0.8336</v>
+      </c>
+      <c r="V4" t="n">
+        <v>0.0321</v>
+      </c>
+      <c r="W4" t="n">
+        <v>46.4</v>
+      </c>
+      <c r="X4" s="4" t="n">
+        <v>0.836</v>
+      </c>
+      <c r="Y4" s="4" t="n">
+        <v>0.9167999999999999</v>
+      </c>
+      <c r="Z4" s="4" t="n">
+        <v>0.9223</v>
+      </c>
+      <c r="AA4" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_epistatic_LINEAR/GB1_epistatic_cv_loss_curves.png</t>
+        </is>
+      </c>
+      <c r="AB4" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_epistatic_LINEAR/GB1_epistatic_predicted_vs_actual_test.png</t>
+        </is>
+      </c>
+      <c r="AC4" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_epistatic_LINEAR/GB1_epistatic_integrated_gradients_heatmap.png</t>
+        </is>
+      </c>
+      <c r="AD4" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_epistatic_LINEAR/GB1_epistatic_integrated_gradients_analysis.png</t>
+        </is>
+      </c>
+      <c r="AE4" t="inlineStr">
+        <is>
+          <t>Will: higher LR and DrpOut</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-04-17 13:58</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>GB1_epistatic</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>python scripts/run_integrated_gradients.py configs/synthetic/GB1_epistatic_config.yaml</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_epistatic_LINEAR/GB1_epistatic_config_snapshot_20260417_135449.yaml</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_epistatic_LINEAR</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_epistatic_LINEAR/GB1_epistatic_run_log_20260417_135240.txt</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>esm_attention</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>128-64-32-16</t>
+        </is>
+      </c>
+      <c r="K5" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0.0005</v>
+      </c>
+      <c r="M5" t="n">
+        <v>64</v>
+      </c>
+      <c r="N5" t="n">
+        <v>50</v>
+      </c>
+      <c r="O5" t="n">
+        <v>10</v>
+      </c>
+      <c r="P5" t="n">
+        <v>15</v>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>huber</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="S5" s="4" t="n">
+        <v>0.7254</v>
+      </c>
+      <c r="T5" t="n">
+        <v>0.016</v>
+      </c>
+      <c r="U5" s="4" t="n">
+        <v>0.8688</v>
+      </c>
+      <c r="V5" t="n">
+        <v>0.0057</v>
+      </c>
+      <c r="W5" t="n">
+        <v>44.6</v>
+      </c>
+      <c r="X5" s="4" t="n">
+        <v>0.8325</v>
+      </c>
+      <c r="Y5" s="4" t="n">
+        <v>0.9127</v>
+      </c>
+      <c r="Z5" s="4" t="n">
+        <v>0.8988</v>
+      </c>
+      <c r="AA5" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_epistatic_LINEAR/GB1_epistatic_cv_loss_curves.png</t>
+        </is>
+      </c>
+      <c r="AB5" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_epistatic_LINEAR/GB1_epistatic_predicted_vs_actual_test.png</t>
+        </is>
+      </c>
+      <c r="AC5" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_epistatic_LINEAR/GB1_epistatic_integrated_gradients_heatmap.png</t>
+        </is>
+      </c>
+      <c r="AD5" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_epistatic_LINEAR/GB1_epistatic_integrated_gradients_analysis.png</t>
+        </is>
+      </c>
+      <c r="AE5" t="inlineStr">
+        <is>
+          <t>Will: lower LR and DrpOut</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2026-04-17 14:04</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>GB1_epistatic</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>python scripts/run_integrated_gradients.py configs/synthetic/GB1_epistatic_config.yaml</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_epistatic_LINEAR/GB1_epistatic_config_snapshot_20260417_135904.yaml</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_epistatic_LINEAR</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_epistatic_LINEAR/GB1_epistatic_run_log_20260417_135904.txt</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>esm_attention</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>128-64-32-16</t>
+        </is>
+      </c>
+      <c r="K6" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0.0005</v>
+      </c>
+      <c r="M6" t="n">
+        <v>64</v>
+      </c>
+      <c r="N6" t="n">
+        <v>50</v>
+      </c>
+      <c r="O6" t="n">
+        <v>10</v>
+      </c>
+      <c r="P6" t="n">
+        <v>15</v>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>huber</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="S6" s="4" t="n">
+        <v>0.7047</v>
+      </c>
+      <c r="T6" t="n">
+        <v>0.0239</v>
+      </c>
+      <c r="U6" s="4" t="n">
+        <v>0.8567</v>
+      </c>
+      <c r="V6" t="n">
+        <v>0.0158</v>
+      </c>
+      <c r="W6" t="n">
+        <v>47</v>
+      </c>
+      <c r="X6" s="4" t="n">
+        <v>0.8169</v>
+      </c>
+      <c r="Y6" s="4" t="n">
+        <v>0.9041</v>
+      </c>
+      <c r="Z6" s="4" t="n">
+        <v>0.8878</v>
+      </c>
+      <c r="AA6" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_epistatic_LINEAR/GB1_epistatic_cv_loss_curves.png</t>
+        </is>
+      </c>
+      <c r="AB6" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_epistatic_LINEAR/GB1_epistatic_predicted_vs_actual_test.png</t>
+        </is>
+      </c>
+      <c r="AC6" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_epistatic_LINEAR/GB1_epistatic_integrated_gradients_heatmap.png</t>
+        </is>
+      </c>
+      <c r="AD6" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_epistatic_LINEAR/GB1_epistatic_integrated_gradients_analysis.png</t>
+        </is>
+      </c>
+      <c r="AE6" t="inlineStr">
+        <is>
+          <t>Will: half initial hidden dims</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H2" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA2" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB2" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC2" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD2" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F3" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H3" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA3" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB3" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC3" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD3" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F4" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H4" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA4" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB4" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC4" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD4" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F5" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H5" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA5" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB5" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC5" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD5" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F6" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA6" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB6" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC6" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD6" r:id="rId30"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2953,7 +4671,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE1"/>
+  <dimension ref="A1:AE6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -3146,7 +4864,649 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2026-04-17 13:17</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>GB1_nonlinear</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>python scripts/run_integrated_gradients.py configs/synthetic/GB1_nonlinear_config.yaml</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_nonlinear_LINEAR/GB1_nonlinear_config_snapshot_20260416_123745.yaml</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_nonlinear_LINEAR</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_nonlinear_LINEAR/GB1_nonlinear_run_log_20260416_123745.txt</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>esm_attention</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>256-128-64-32</t>
+        </is>
+      </c>
+      <c r="K2" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="M2" t="n">
+        <v>64</v>
+      </c>
+      <c r="N2" t="n">
+        <v>50</v>
+      </c>
+      <c r="O2" t="n">
+        <v>10</v>
+      </c>
+      <c r="P2" t="n">
+        <v>15</v>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>huber</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="S2" s="4" t="n">
+        <v>0.7554999999999999</v>
+      </c>
+      <c r="T2" t="n">
+        <v>0.0163</v>
+      </c>
+      <c r="U2" s="4" t="n">
+        <v>0.8843</v>
+      </c>
+      <c r="V2" t="n">
+        <v>0.009299999999999999</v>
+      </c>
+      <c r="W2" t="n">
+        <v>45.4</v>
+      </c>
+      <c r="X2" s="4" t="n">
+        <v>0.8066</v>
+      </c>
+      <c r="Y2" s="4" t="n">
+        <v>0.8996</v>
+      </c>
+      <c r="Z2" s="4" t="n">
+        <v>0.9005</v>
+      </c>
+      <c r="AA2" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_nonlinear_LINEAR/GB1_nonlinear_cv_loss_curves.png</t>
+        </is>
+      </c>
+      <c r="AB2" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_nonlinear_LINEAR/GB1_nonlinear_predicted_vs_actual_test.png</t>
+        </is>
+      </c>
+      <c r="AC2" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_nonlinear_LINEAR/GB1_nonlinear_integrated_gradients_heatmap.png</t>
+        </is>
+      </c>
+      <c r="AD2" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_nonlinear_LINEAR/GB1_nonlinear_integrated_gradients_analysis.png</t>
+        </is>
+      </c>
+      <c r="AE2" t="inlineStr">
+        <is>
+          <t>Will: initial run</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-04-17 13:36</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>GB1_nonlinear</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>python scripts/run_integrated_gradients.py configs/synthetic/GB1_nonlinear_config.yaml</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_nonlinear_LINEAR/GB1_nonlinear_config_snapshot_20260417_133148.yaml</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_nonlinear_LINEAR</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_nonlinear_LINEAR/GB1_nonlinear_run_log_20260417_133148.txt</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>esm_attention</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>512-256-128-64</t>
+        </is>
+      </c>
+      <c r="K3" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="M3" t="n">
+        <v>64</v>
+      </c>
+      <c r="N3" t="n">
+        <v>50</v>
+      </c>
+      <c r="O3" t="n">
+        <v>10</v>
+      </c>
+      <c r="P3" t="n">
+        <v>15</v>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>huber</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="S3" s="4" t="n">
+        <v>0.7586000000000001</v>
+      </c>
+      <c r="T3" t="n">
+        <v>0.0268</v>
+      </c>
+      <c r="U3" s="4" t="n">
+        <v>0.8848</v>
+      </c>
+      <c r="V3" t="n">
+        <v>0.0197</v>
+      </c>
+      <c r="W3" t="n">
+        <v>45.4</v>
+      </c>
+      <c r="X3" s="4" t="n">
+        <v>0.7991</v>
+      </c>
+      <c r="Y3" s="4" t="n">
+        <v>0.8942</v>
+      </c>
+      <c r="Z3" s="4" t="n">
+        <v>0.8804</v>
+      </c>
+      <c r="AA3" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_nonlinear_LINEAR/GB1_nonlinear_cv_loss_curves.png</t>
+        </is>
+      </c>
+      <c r="AB3" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_nonlinear_LINEAR/GB1_nonlinear_predicted_vs_actual_test.png</t>
+        </is>
+      </c>
+      <c r="AC3" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_nonlinear_LINEAR/GB1_nonlinear_integrated_gradients_heatmap.png</t>
+        </is>
+      </c>
+      <c r="AD3" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_nonlinear_LINEAR/GB1_nonlinear_integrated_gradients_analysis.png</t>
+        </is>
+      </c>
+      <c r="AE3" t="inlineStr">
+        <is>
+          <t>Will: Double hidden dims</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-04-17 13:51</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>GB1_nonlinear</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>python scripts/run_integrated_gradients.py configs/synthetic/GB1_nonlinear_config.yaml</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_nonlinear_LINEAR/GB1_nonlinear_config_snapshot_20260417_134434.yaml</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_nonlinear_LINEAR</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_nonlinear_LINEAR/GB1_nonlinear_run_log_20260417_134434.txt</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>esm_attention</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>512-256-128-64</t>
+        </is>
+      </c>
+      <c r="K4" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="M4" t="n">
+        <v>64</v>
+      </c>
+      <c r="N4" t="n">
+        <v>50</v>
+      </c>
+      <c r="O4" t="n">
+        <v>10</v>
+      </c>
+      <c r="P4" t="n">
+        <v>15</v>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>huber</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="S4" s="4" t="n">
+        <v>0.5883</v>
+      </c>
+      <c r="T4" t="n">
+        <v>0.0663</v>
+      </c>
+      <c r="U4" s="4" t="n">
+        <v>0.7996</v>
+      </c>
+      <c r="V4" t="n">
+        <v>0.0408</v>
+      </c>
+      <c r="W4" t="n">
+        <v>41.4</v>
+      </c>
+      <c r="X4" s="4" t="n">
+        <v>0.7616000000000001</v>
+      </c>
+      <c r="Y4" s="4" t="n">
+        <v>0.8749</v>
+      </c>
+      <c r="Z4" s="4" t="n">
+        <v>0.8973</v>
+      </c>
+      <c r="AA4" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_nonlinear_LINEAR/GB1_nonlinear_cv_loss_curves.png</t>
+        </is>
+      </c>
+      <c r="AB4" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_nonlinear_LINEAR/GB1_nonlinear_predicted_vs_actual_test.png</t>
+        </is>
+      </c>
+      <c r="AC4" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_nonlinear_LINEAR/GB1_nonlinear_integrated_gradients_heatmap.png</t>
+        </is>
+      </c>
+      <c r="AD4" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_nonlinear_LINEAR/GB1_nonlinear_integrated_gradients_analysis.png</t>
+        </is>
+      </c>
+      <c r="AE4" t="inlineStr">
+        <is>
+          <t>Will: higher LR and DrpOut</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-04-17 13:58</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>GB1_nonlinear</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>python scripts/run_integrated_gradients.py configs/synthetic/GB1_nonlinear_config.yaml</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_nonlinear_LINEAR/GB1_nonlinear_config_snapshot_20260417_135447.yaml</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_nonlinear_LINEAR</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_nonlinear_LINEAR/GB1_nonlinear_run_log_20260417_135241.txt</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>esm_attention</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>128-64-32-16</t>
+        </is>
+      </c>
+      <c r="K5" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0.0005</v>
+      </c>
+      <c r="M5" t="n">
+        <v>64</v>
+      </c>
+      <c r="N5" t="n">
+        <v>50</v>
+      </c>
+      <c r="O5" t="n">
+        <v>10</v>
+      </c>
+      <c r="P5" t="n">
+        <v>15</v>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>huber</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="S5" s="4" t="n">
+        <v>0.7433</v>
+      </c>
+      <c r="T5" t="n">
+        <v>0.0212</v>
+      </c>
+      <c r="U5" s="4" t="n">
+        <v>0.8748</v>
+      </c>
+      <c r="V5" t="n">
+        <v>0.0127</v>
+      </c>
+      <c r="W5" t="n">
+        <v>47.6</v>
+      </c>
+      <c r="X5" s="4" t="n">
+        <v>0.8115</v>
+      </c>
+      <c r="Y5" s="4" t="n">
+        <v>0.9012</v>
+      </c>
+      <c r="Z5" s="4" t="n">
+        <v>0.8848</v>
+      </c>
+      <c r="AA5" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_nonlinear_LINEAR/GB1_nonlinear_cv_loss_curves.png</t>
+        </is>
+      </c>
+      <c r="AB5" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_nonlinear_LINEAR/GB1_nonlinear_predicted_vs_actual_test.png</t>
+        </is>
+      </c>
+      <c r="AC5" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_nonlinear_LINEAR/GB1_nonlinear_integrated_gradients_heatmap.png</t>
+        </is>
+      </c>
+      <c r="AD5" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_nonlinear_LINEAR/GB1_nonlinear_integrated_gradients_analysis.png</t>
+        </is>
+      </c>
+      <c r="AE5" t="inlineStr">
+        <is>
+          <t>Will: lower LR and DrpOut</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2026-04-17 14:04</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>GB1_nonlinear</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>python scripts/run_integrated_gradients.py configs/synthetic/GB1_nonlinear_config.yaml</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_nonlinear_LINEAR/GB1_nonlinear_config_snapshot_20260417_135908.yaml</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_nonlinear_LINEAR</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_nonlinear_LINEAR/GB1_nonlinear_run_log_20260417_135908.txt</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>esm_attention</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>128-64-32-16</t>
+        </is>
+      </c>
+      <c r="K6" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0.0005</v>
+      </c>
+      <c r="M6" t="n">
+        <v>64</v>
+      </c>
+      <c r="N6" t="n">
+        <v>50</v>
+      </c>
+      <c r="O6" t="n">
+        <v>10</v>
+      </c>
+      <c r="P6" t="n">
+        <v>15</v>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>huber</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="S6" s="4" t="n">
+        <v>0.6952</v>
+      </c>
+      <c r="T6" t="n">
+        <v>0.0324</v>
+      </c>
+      <c r="U6" s="4" t="n">
+        <v>0.847</v>
+      </c>
+      <c r="V6" t="n">
+        <v>0.0126</v>
+      </c>
+      <c r="W6" t="n">
+        <v>47.8</v>
+      </c>
+      <c r="X6" s="4" t="n">
+        <v>0.7498</v>
+      </c>
+      <c r="Y6" s="4" t="n">
+        <v>0.8693</v>
+      </c>
+      <c r="Z6" s="4" t="n">
+        <v>0.8617</v>
+      </c>
+      <c r="AA6" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_nonlinear_LINEAR/GB1_nonlinear_cv_loss_curves.png</t>
+        </is>
+      </c>
+      <c r="AB6" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_nonlinear_LINEAR/GB1_nonlinear_predicted_vs_actual_test.png</t>
+        </is>
+      </c>
+      <c r="AC6" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_nonlinear_LINEAR/GB1_nonlinear_integrated_gradients_heatmap.png</t>
+        </is>
+      </c>
+      <c r="AD6" s="3" t="inlineStr">
+        <is>
+          <t>results/synthetic/GB1_nonlinear_LINEAR/GB1_nonlinear_integrated_gradients_analysis.png</t>
+        </is>
+      </c>
+      <c r="AE6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Will: half initial hidden dims </t>
+        </is>
+      </c>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H2" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA2" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB2" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC2" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD2" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F3" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H3" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA3" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB3" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC3" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD3" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F4" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H4" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA4" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB4" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC4" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD4" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F5" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H5" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA5" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB5" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC5" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD5" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F6" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA6" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB6" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC6" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD6" r:id="rId30"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Revert "synth GB1  LINEAR results"
This reverts commit 4ce347f2e9b6f8a99639c224b3631991ff80e7c0.
</commit_message>
<xml_diff>
--- a/experiment_tracker.xlsx
+++ b/experiment_tracker.xlsx
@@ -1021,6 +1021,7 @@
           <t>python scripts/run_integrated_gradients.py configs/synthetic/T4Lysozyme_nonlinear_config.yaml</t>
         </is>
       </c>
+      <c r="E2" t="inlineStr"/>
       <c r="F2" s="3" t="inlineStr">
         <is>
           <t>results/synthetic/T4Lysozyme_nonlinear_LINEAR/T4Lysozyme_nonlinear_config_snapshot_20260414_201415.yaml</t>
@@ -2014,7 +2015,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -2069,18 +2070,18 @@
           <t>GB1_additive</t>
         </is>
       </c>
-      <c r="B2" s="4" t="n">
-        <v>0.8463000000000001</v>
-      </c>
-      <c r="C2" s="4" t="n">
-        <v>0.9134</v>
+      <c r="B2" s="2" t="n">
+        <v>-0.0425</v>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>-0.06560000000000001</v>
       </c>
       <c r="D2" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-04-17 13:34</t>
+          <t>2026-04-10 18:24</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -2262,58 +2263,6 @@
       <c r="F9" t="inlineStr">
         <is>
           <t>results/synthetic/T4Lysozyme_nonlinear_LINEAR</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>GB1_epistatic</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="n">
-        <v>0.8379</v>
-      </c>
-      <c r="C10" s="4" t="n">
-        <v>0.8935</v>
-      </c>
-      <c r="D10" t="n">
-        <v>5</v>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>2026-04-17 13:36</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_epistatic_LINEAR</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>GB1_nonlinear</t>
-        </is>
-      </c>
-      <c r="B11" s="4" t="n">
-        <v>0.8115</v>
-      </c>
-      <c r="C11" s="4" t="n">
-        <v>0.8848</v>
-      </c>
-      <c r="D11" t="n">
-        <v>5</v>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>2026-04-17 13:58</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_nonlinear_LINEAR</t>
         </is>
       </c>
     </row>
@@ -2328,7 +2277,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE11"/>
+  <dimension ref="A1:AE3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -2775,982 +2724,6 @@
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>2026-04-16 11:59</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>GB1_additive</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>python scripts/run_integrated_gradients.py configs/synthetic/GB1_additive_config.yaml</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_additive_LINEAR/GB1_additive_config_snapshot_20260415_145841.yaml</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_additive_LINEAR</t>
-        </is>
-      </c>
-      <c r="H4" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_additive_LINEAR/GB1_additive_run_log_20260415_145840.txt</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>esm_attention</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>256-128-64-32</t>
-        </is>
-      </c>
-      <c r="K4" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="L4" t="n">
-        <v>0.001</v>
-      </c>
-      <c r="M4" t="n">
-        <v>64</v>
-      </c>
-      <c r="N4" t="n">
-        <v>50</v>
-      </c>
-      <c r="O4" t="n">
-        <v>10</v>
-      </c>
-      <c r="P4" t="n">
-        <v>15</v>
-      </c>
-      <c r="Q4" t="inlineStr">
-        <is>
-          <t>huber</t>
-        </is>
-      </c>
-      <c r="R4" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="S4" s="4" t="n">
-        <v>0.7449</v>
-      </c>
-      <c r="T4" t="n">
-        <v>0.022</v>
-      </c>
-      <c r="U4" s="4" t="n">
-        <v>0.8656</v>
-      </c>
-      <c r="V4" t="n">
-        <v>0.0074</v>
-      </c>
-      <c r="W4" t="n">
-        <v>45.4</v>
-      </c>
-      <c r="X4" s="4" t="n">
-        <v>0.83</v>
-      </c>
-      <c r="Y4" s="4" t="n">
-        <v>0.9117</v>
-      </c>
-      <c r="Z4" s="4" t="n">
-        <v>0.8874</v>
-      </c>
-      <c r="AA4" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_additive_LINEAR/GB1_additive_cv_loss_curves.png</t>
-        </is>
-      </c>
-      <c r="AB4" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_additive_LINEAR/GB1_additive_predicted_vs_actual_test.png</t>
-        </is>
-      </c>
-      <c r="AC4" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_additive_LINEAR/GB1_additive_integrated_gradients_heatmap.png</t>
-        </is>
-      </c>
-      <c r="AD4" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_additive_LINEAR/GB1_additive_integrated_gradients_analysis.png</t>
-        </is>
-      </c>
-      <c r="AE4" t="inlineStr">
-        <is>
-          <t>Will: initial run</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="n">
-        <v>4</v>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>2026-04-16 12:20</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>GB1_additive</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>python scripts/run_integrated_gradients.py configs/synthetic/GB1_additive_config.yaml</t>
-        </is>
-      </c>
-      <c r="F5" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_additive_LINEAR/GB1_additive_config_snapshot_20260415_145841.yaml</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_additive_LINEAR</t>
-        </is>
-      </c>
-      <c r="H5" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_additive_LINEAR/GB1_additive_run_log_20260415_145840.txt</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>esm_attention</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>256-128-64-32</t>
-        </is>
-      </c>
-      <c r="K5" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="L5" t="n">
-        <v>0.001</v>
-      </c>
-      <c r="M5" t="n">
-        <v>64</v>
-      </c>
-      <c r="N5" t="n">
-        <v>50</v>
-      </c>
-      <c r="O5" t="n">
-        <v>10</v>
-      </c>
-      <c r="P5" t="n">
-        <v>15</v>
-      </c>
-      <c r="Q5" t="inlineStr">
-        <is>
-          <t>huber</t>
-        </is>
-      </c>
-      <c r="R5" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="S5" s="4" t="n">
-        <v>0.7449</v>
-      </c>
-      <c r="T5" t="n">
-        <v>0.022</v>
-      </c>
-      <c r="U5" s="4" t="n">
-        <v>0.8656</v>
-      </c>
-      <c r="V5" t="n">
-        <v>0.0074</v>
-      </c>
-      <c r="W5" t="n">
-        <v>45.4</v>
-      </c>
-      <c r="X5" s="4" t="n">
-        <v>0.83</v>
-      </c>
-      <c r="Y5" s="4" t="n">
-        <v>0.9117</v>
-      </c>
-      <c r="Z5" s="4" t="n">
-        <v>0.8874</v>
-      </c>
-      <c r="AA5" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_additive_LINEAR/GB1_additive_cv_loss_curves.png</t>
-        </is>
-      </c>
-      <c r="AB5" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_additive_LINEAR/GB1_additive_predicted_vs_actual_test.png</t>
-        </is>
-      </c>
-      <c r="AC5" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_additive_LINEAR/GB1_additive_integrated_gradients_heatmap.png</t>
-        </is>
-      </c>
-      <c r="AD5" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_additive_LINEAR/GB1_additive_integrated_gradients_analysis.png</t>
-        </is>
-      </c>
-      <c r="AE5" t="inlineStr">
-        <is>
-          <t>Will: initial run</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="n">
-        <v>5</v>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>2026-04-16 12:36</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>GB1_additive</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>python scripts/run_integrated_gradients.py configs/synthetic/GB1_additive_config.yaml</t>
-        </is>
-      </c>
-      <c r="F6" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_additive_LINEAR/GB1_additive_config_snapshot_20260416_122524.yaml</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_additive_LINEAR</t>
-        </is>
-      </c>
-      <c r="H6" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_additive_LINEAR/GB1_additive_run_log_20260416_122524.txt</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>esm_attention</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>512-256-128-64</t>
-        </is>
-      </c>
-      <c r="K6" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="L6" t="n">
-        <v>0.001</v>
-      </c>
-      <c r="M6" t="n">
-        <v>64</v>
-      </c>
-      <c r="N6" t="n">
-        <v>50</v>
-      </c>
-      <c r="O6" t="n">
-        <v>10</v>
-      </c>
-      <c r="P6" t="n">
-        <v>15</v>
-      </c>
-      <c r="Q6" t="inlineStr">
-        <is>
-          <t>huber</t>
-        </is>
-      </c>
-      <c r="R6" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="S6" s="4" t="n">
-        <v>0.7717000000000001</v>
-      </c>
-      <c r="T6" t="n">
-        <v>0.0302</v>
-      </c>
-      <c r="U6" s="4" t="n">
-        <v>0.8875</v>
-      </c>
-      <c r="V6" t="n">
-        <v>0.0117</v>
-      </c>
-      <c r="W6" t="n">
-        <v>47.2</v>
-      </c>
-      <c r="X6" s="4" t="n">
-        <v>0.842</v>
-      </c>
-      <c r="Y6" s="4" t="n">
-        <v>0.9177</v>
-      </c>
-      <c r="Z6" s="4" t="n">
-        <v>0.8997000000000001</v>
-      </c>
-      <c r="AA6" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_additive_LINEAR/GB1_additive_cv_loss_curves.png</t>
-        </is>
-      </c>
-      <c r="AB6" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_additive_LINEAR/GB1_additive_predicted_vs_actual_test.png</t>
-        </is>
-      </c>
-      <c r="AC6" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_additive_LINEAR/GB1_additive_integrated_gradients_heatmap.png</t>
-        </is>
-      </c>
-      <c r="AD6" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_additive_LINEAR/GB1_additive_integrated_gradients_analysis.png</t>
-        </is>
-      </c>
-      <c r="AE6" t="inlineStr">
-        <is>
-          <t>Will: doubled hidden dimensions</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="n">
-        <v>6</v>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>2026-04-17 13:34</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>GB1_additive</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>python scripts/run_integrated_gradients.py configs/synthetic/GB1_additive_config.yaml</t>
-        </is>
-      </c>
-      <c r="F7" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_additive_LINEAR/GB1_additive_config_snapshot_20260417_132916.yaml</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_additive_LINEAR</t>
-        </is>
-      </c>
-      <c r="H7" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_additive_LINEAR/GB1_additive_run_log_20260417_132915.txt</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>esm_attention</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>512-256-128-64</t>
-        </is>
-      </c>
-      <c r="K7" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="L7" t="n">
-        <v>0.005</v>
-      </c>
-      <c r="M7" t="n">
-        <v>64</v>
-      </c>
-      <c r="N7" t="n">
-        <v>50</v>
-      </c>
-      <c r="O7" t="n">
-        <v>10</v>
-      </c>
-      <c r="P7" t="n">
-        <v>15</v>
-      </c>
-      <c r="Q7" t="inlineStr">
-        <is>
-          <t>huber</t>
-        </is>
-      </c>
-      <c r="R7" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="S7" s="4" t="n">
-        <v>0.6127</v>
-      </c>
-      <c r="T7" t="n">
-        <v>0.0822</v>
-      </c>
-      <c r="U7" s="4" t="n">
-        <v>0.8051</v>
-      </c>
-      <c r="V7" t="n">
-        <v>0.0466</v>
-      </c>
-      <c r="W7" t="n">
-        <v>45</v>
-      </c>
-      <c r="X7" s="4" t="n">
-        <v>0.8463000000000001</v>
-      </c>
-      <c r="Y7" s="4" t="n">
-        <v>0.9225</v>
-      </c>
-      <c r="Z7" s="4" t="n">
-        <v>0.9134</v>
-      </c>
-      <c r="AA7" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_additive_LINEAR/GB1_additive_cv_loss_curves.png</t>
-        </is>
-      </c>
-      <c r="AB7" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_additive_LINEAR/GB1_additive_predicted_vs_actual_test.png</t>
-        </is>
-      </c>
-      <c r="AC7" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_additive_LINEAR/GB1_additive_integrated_gradients_heatmap.png</t>
-        </is>
-      </c>
-      <c r="AD7" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_additive_LINEAR/GB1_additive_integrated_gradients_analysis.png</t>
-        </is>
-      </c>
-      <c r="AE7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Will:Higer LR &amp; DrpOut </t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="n">
-        <v>7</v>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>2026-04-17 13:39</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>GB1_additive</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>python scripts/run_integrated_gradients.py configs/synthetic/GB1_additive_config.yaml</t>
-        </is>
-      </c>
-      <c r="F8" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_additive_LINEAR/GB1_additive_config_snapshot_20260417_133447.yaml</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_additive_LINEAR</t>
-        </is>
-      </c>
-      <c r="H8" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_additive_LINEAR/GB1_additive_run_log_20260417_133447.txt</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>esm_attention</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>512-256-128-64</t>
-        </is>
-      </c>
-      <c r="K8" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="L8" t="n">
-        <v>0.0005</v>
-      </c>
-      <c r="M8" t="n">
-        <v>64</v>
-      </c>
-      <c r="N8" t="n">
-        <v>50</v>
-      </c>
-      <c r="O8" t="n">
-        <v>10</v>
-      </c>
-      <c r="P8" t="n">
-        <v>15</v>
-      </c>
-      <c r="Q8" t="inlineStr">
-        <is>
-          <t>huber</t>
-        </is>
-      </c>
-      <c r="R8" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="S8" s="4" t="n">
-        <v>0.7517</v>
-      </c>
-      <c r="T8" t="n">
-        <v>0.0222</v>
-      </c>
-      <c r="U8" s="4" t="n">
-        <v>0.8774999999999999</v>
-      </c>
-      <c r="V8" t="n">
-        <v>0.0077</v>
-      </c>
-      <c r="W8" t="n">
-        <v>46.4</v>
-      </c>
-      <c r="X8" s="4" t="n">
-        <v>0.8178</v>
-      </c>
-      <c r="Y8" s="4" t="n">
-        <v>0.9049</v>
-      </c>
-      <c r="Z8" s="4" t="n">
-        <v>0.8802</v>
-      </c>
-      <c r="AA8" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_additive_LINEAR/GB1_additive_cv_loss_curves.png</t>
-        </is>
-      </c>
-      <c r="AB8" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_additive_LINEAR/GB1_additive_predicted_vs_actual_test.png</t>
-        </is>
-      </c>
-      <c r="AC8" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_additive_LINEAR/GB1_additive_integrated_gradients_heatmap.png</t>
-        </is>
-      </c>
-      <c r="AD8" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_additive_LINEAR/GB1_additive_integrated_gradients_analysis.png</t>
-        </is>
-      </c>
-      <c r="AE8" t="inlineStr">
-        <is>
-          <t>Will: Lower LR and DrpOut</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="n">
-        <v>8</v>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>2026-04-17 13:47</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>GB1_additive</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>python scripts/run_integrated_gradients.py configs/synthetic/GB1_additive_config.yaml</t>
-        </is>
-      </c>
-      <c r="F9" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_additive_LINEAR/GB1_additive_config_snapshot_20260417_134320.yaml</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_additive_LINEAR</t>
-        </is>
-      </c>
-      <c r="H9" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_additive_LINEAR/GB1_additive_run_log_20260417_134319.txt</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>esm_attention</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>128-64-32-16</t>
-        </is>
-      </c>
-      <c r="K9" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="L9" t="n">
-        <v>0.0005</v>
-      </c>
-      <c r="M9" t="n">
-        <v>64</v>
-      </c>
-      <c r="N9" t="n">
-        <v>50</v>
-      </c>
-      <c r="O9" t="n">
-        <v>10</v>
-      </c>
-      <c r="P9" t="n">
-        <v>15</v>
-      </c>
-      <c r="Q9" t="inlineStr">
-        <is>
-          <t>huber</t>
-        </is>
-      </c>
-      <c r="R9" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="S9" s="4" t="n">
-        <v>0.7143</v>
-      </c>
-      <c r="T9" t="n">
-        <v>0.0258</v>
-      </c>
-      <c r="U9" s="4" t="n">
-        <v>0.8561</v>
-      </c>
-      <c r="V9" t="n">
-        <v>0.008999999999999999</v>
-      </c>
-      <c r="W9" t="n">
-        <v>47.4</v>
-      </c>
-      <c r="X9" s="4" t="n">
-        <v>0.8067</v>
-      </c>
-      <c r="Y9" s="4" t="n">
-        <v>0.8986</v>
-      </c>
-      <c r="Z9" s="4" t="n">
-        <v>0.8751</v>
-      </c>
-      <c r="AA9" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_additive_LINEAR/GB1_additive_cv_loss_curves.png</t>
-        </is>
-      </c>
-      <c r="AB9" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_additive_LINEAR/GB1_additive_predicted_vs_actual_test.png</t>
-        </is>
-      </c>
-      <c r="AC9" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_additive_LINEAR/GB1_additive_integrated_gradients_heatmap.png</t>
-        </is>
-      </c>
-      <c r="AD9" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_additive_LINEAR/GB1_additive_integrated_gradients_analysis.png</t>
-        </is>
-      </c>
-      <c r="AE9" t="inlineStr">
-        <is>
-          <t>Will: half initial hidden dims</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="n">
-        <v>9</v>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>2026-04-17 13:50</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>GB1_additive</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>python scripts/run_integrated_gradients.py configs/synthetic/GB1_additive_config.yaml</t>
-        </is>
-      </c>
-      <c r="F10" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_additive_LINEAR/GB1_additive_config_snapshot_20260417_134830.yaml</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_additive_LINEAR</t>
-        </is>
-      </c>
-      <c r="H10" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_additive_LINEAR/GB1_additive_run_log_20260417_134829.txt</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>esm_attention</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>128-64-32-16</t>
-        </is>
-      </c>
-      <c r="K10" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="L10" t="n">
-        <v>0.001</v>
-      </c>
-      <c r="M10" t="n">
-        <v>64</v>
-      </c>
-      <c r="N10" t="n">
-        <v>50</v>
-      </c>
-      <c r="O10" t="n">
-        <v>10</v>
-      </c>
-      <c r="P10" t="n">
-        <v>15</v>
-      </c>
-      <c r="Q10" t="inlineStr">
-        <is>
-          <t>huber</t>
-        </is>
-      </c>
-      <c r="R10" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="S10" s="4" t="n">
-        <v>0.7143</v>
-      </c>
-      <c r="T10" t="n">
-        <v>0.0258</v>
-      </c>
-      <c r="U10" s="4" t="n">
-        <v>0.8561</v>
-      </c>
-      <c r="V10" t="n">
-        <v>0.008999999999999999</v>
-      </c>
-      <c r="W10" t="n">
-        <v>47.4</v>
-      </c>
-      <c r="X10" s="4" t="n">
-        <v>0.8067</v>
-      </c>
-      <c r="Y10" s="4" t="n">
-        <v>0.8986</v>
-      </c>
-      <c r="Z10" s="4" t="n">
-        <v>0.8751</v>
-      </c>
-      <c r="AA10" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_additive_LINEAR/GB1_additive_cv_loss_curves.png</t>
-        </is>
-      </c>
-      <c r="AB10" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_additive_LINEAR/GB1_additive_predicted_vs_actual_test.png</t>
-        </is>
-      </c>
-      <c r="AC10" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_additive_LINEAR/GB1_additive_integrated_gradients_heatmap.png</t>
-        </is>
-      </c>
-      <c r="AD10" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_additive_LINEAR/GB1_additive_integrated_gradients_analysis.png</t>
-        </is>
-      </c>
-      <c r="AE10" t="inlineStr">
-        <is>
-          <t>Will: higher LR and DrpOut</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="n">
-        <v>10</v>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>2026-04-17 13:53</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>GB1_additive</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>python scripts/run_integrated_gradients.py configs/synthetic/GB1_additive_config.yaml</t>
-        </is>
-      </c>
-      <c r="F11" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_additive_LINEAR/GB1_additive_config_snapshot_20260417_134830.yaml</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_additive_LINEAR</t>
-        </is>
-      </c>
-      <c r="H11" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_additive_LINEAR/GB1_additive_run_log_20260417_134829.txt</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>esm_attention</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>128-64-32-16</t>
-        </is>
-      </c>
-      <c r="K11" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="L11" t="n">
-        <v>0.001</v>
-      </c>
-      <c r="M11" t="n">
-        <v>64</v>
-      </c>
-      <c r="N11" t="n">
-        <v>50</v>
-      </c>
-      <c r="O11" t="n">
-        <v>10</v>
-      </c>
-      <c r="P11" t="n">
-        <v>15</v>
-      </c>
-      <c r="Q11" t="inlineStr">
-        <is>
-          <t>huber</t>
-        </is>
-      </c>
-      <c r="R11" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="S11" s="4" t="n">
-        <v>0.7615</v>
-      </c>
-      <c r="T11" t="n">
-        <v>0.0135</v>
-      </c>
-      <c r="U11" s="4" t="n">
-        <v>0.8819</v>
-      </c>
-      <c r="V11" t="n">
-        <v>0.0102</v>
-      </c>
-      <c r="W11" t="n">
-        <v>47.4</v>
-      </c>
-      <c r="X11" s="4" t="n">
-        <v>0.8137</v>
-      </c>
-      <c r="Y11" s="4" t="n">
-        <v>0.905</v>
-      </c>
-      <c r="Z11" s="4" t="n">
-        <v>0.8871</v>
-      </c>
-      <c r="AA11" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_additive_LINEAR/GB1_additive_cv_loss_curves.png</t>
-        </is>
-      </c>
-      <c r="AB11" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_additive_LINEAR/GB1_additive_predicted_vs_actual_test.png</t>
-        </is>
-      </c>
-      <c r="AC11" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_additive_LINEAR/GB1_additive_integrated_gradients_heatmap.png</t>
-        </is>
-      </c>
-      <c r="AD11" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_additive_LINEAR/GB1_additive_integrated_gradients_analysis.png</t>
-        </is>
-      </c>
-      <c r="AE11" t="inlineStr">
-        <is>
-          <t>Will: normal LR and DrpOut</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F2" r:id="rId1"/>
@@ -3765,54 +2738,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB3" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC3" r:id="rId11"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD3" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F4" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H4" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA4" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB4" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC4" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD4" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F5" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H5" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA5" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB5" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC5" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD5" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F6" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA6" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB6" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC6" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD6" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F7" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H7" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA7" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB7" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC7" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD7" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H8" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA8" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB8" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC8" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD8" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F9" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H9" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA9" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB9" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC9" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD9" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F10" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H10" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA10" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB10" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC10" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD10" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F11" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H11" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA11" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB11" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC11" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD11" r:id="rId60"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3824,7 +2749,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE6"/>
+  <dimension ref="A1:AE1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -4017,650 +2942,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>2026-04-17 13:17</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>GB1_epistatic</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>python scripts/run_integrated_gradients.py configs/synthetic/GB1_epistatic_config.yaml</t>
-        </is>
-      </c>
-      <c r="F2" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_epistatic_LINEAR/GB1_epistatic_config_snapshot_20260416_123720.yaml</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_epistatic_LINEAR</t>
-        </is>
-      </c>
-      <c r="H2" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_epistatic_LINEAR/GB1_epistatic_run_log_20260416_123720.txt</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>esm_attention</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>256-128-64-32</t>
-        </is>
-      </c>
-      <c r="K2" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="L2" t="n">
-        <v>0.001</v>
-      </c>
-      <c r="M2" t="n">
-        <v>64</v>
-      </c>
-      <c r="N2" t="n">
-        <v>50</v>
-      </c>
-      <c r="O2" t="n">
-        <v>10</v>
-      </c>
-      <c r="P2" t="n">
-        <v>15</v>
-      </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>huber</t>
-        </is>
-      </c>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="S2" s="4" t="n">
-        <v>0.7529</v>
-      </c>
-      <c r="T2" t="n">
-        <v>0.0277</v>
-      </c>
-      <c r="U2" s="4" t="n">
-        <v>0.8811</v>
-      </c>
-      <c r="V2" t="n">
-        <v>0.0124</v>
-      </c>
-      <c r="W2" t="n">
-        <v>44.2</v>
-      </c>
-      <c r="X2" s="4" t="n">
-        <v>0.8237</v>
-      </c>
-      <c r="Y2" s="4" t="n">
-        <v>0.9079</v>
-      </c>
-      <c r="Z2" s="4" t="n">
-        <v>0.8924</v>
-      </c>
-      <c r="AA2" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_epistatic_LINEAR/GB1_epistatic_cv_loss_curves.png</t>
-        </is>
-      </c>
-      <c r="AB2" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_epistatic_LINEAR/GB1_epistatic_predicted_vs_actual_test.png</t>
-        </is>
-      </c>
-      <c r="AC2" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_epistatic_LINEAR/GB1_epistatic_integrated_gradients_heatmap.png</t>
-        </is>
-      </c>
-      <c r="AD2" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_epistatic_LINEAR/GB1_epistatic_integrated_gradients_analysis.png</t>
-        </is>
-      </c>
-      <c r="AE2" t="inlineStr">
-        <is>
-          <t>Will: initial run</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>2026-04-17 13:36</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>GB1_epistatic</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>python scripts/run_integrated_gradients.py configs/synthetic/GB1_epistatic_config.yaml</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_epistatic_LINEAR/GB1_epistatic_config_snapshot_20260417_133023.yaml</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_epistatic_LINEAR</t>
-        </is>
-      </c>
-      <c r="H3" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_epistatic_LINEAR/GB1_epistatic_run_log_20260417_133023.txt</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>esm_attention</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>512-256-128-64</t>
-        </is>
-      </c>
-      <c r="K3" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="L3" t="n">
-        <v>0.001</v>
-      </c>
-      <c r="M3" t="n">
-        <v>64</v>
-      </c>
-      <c r="N3" t="n">
-        <v>50</v>
-      </c>
-      <c r="O3" t="n">
-        <v>10</v>
-      </c>
-      <c r="P3" t="n">
-        <v>15</v>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>huber</t>
-        </is>
-      </c>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="S3" s="4" t="n">
-        <v>0.7327</v>
-      </c>
-      <c r="T3" t="n">
-        <v>0.052</v>
-      </c>
-      <c r="U3" s="4" t="n">
-        <v>0.8614000000000001</v>
-      </c>
-      <c r="V3" t="n">
-        <v>0.0201</v>
-      </c>
-      <c r="W3" t="n">
-        <v>47.4</v>
-      </c>
-      <c r="X3" s="4" t="n">
-        <v>0.8379</v>
-      </c>
-      <c r="Y3" s="4" t="n">
-        <v>0.9155</v>
-      </c>
-      <c r="Z3" s="4" t="n">
-        <v>0.8935</v>
-      </c>
-      <c r="AA3" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_epistatic_LINEAR/GB1_epistatic_cv_loss_curves.png</t>
-        </is>
-      </c>
-      <c r="AB3" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_epistatic_LINEAR/GB1_epistatic_predicted_vs_actual_test.png</t>
-        </is>
-      </c>
-      <c r="AC3" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_epistatic_LINEAR/GB1_epistatic_integrated_gradients_heatmap.png</t>
-        </is>
-      </c>
-      <c r="AD3" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_epistatic_LINEAR/GB1_epistatic_integrated_gradients_analysis.png</t>
-        </is>
-      </c>
-      <c r="AE3" t="inlineStr">
-        <is>
-          <t>Will: Double hidden dims</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>2026-04-17 13:51</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>GB1_epistatic</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>python scripts/run_integrated_gradients.py configs/synthetic/GB1_epistatic_config.yaml</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_epistatic_LINEAR/GB1_epistatic_config_snapshot_20260417_134425.yaml</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_epistatic_LINEAR</t>
-        </is>
-      </c>
-      <c r="H4" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_epistatic_LINEAR/GB1_epistatic_run_log_20260417_134425.txt</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>esm_attention</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>512-256-128-64</t>
-        </is>
-      </c>
-      <c r="K4" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="L4" t="n">
-        <v>0.005</v>
-      </c>
-      <c r="M4" t="n">
-        <v>64</v>
-      </c>
-      <c r="N4" t="n">
-        <v>50</v>
-      </c>
-      <c r="O4" t="n">
-        <v>10</v>
-      </c>
-      <c r="P4" t="n">
-        <v>15</v>
-      </c>
-      <c r="Q4" t="inlineStr">
-        <is>
-          <t>huber</t>
-        </is>
-      </c>
-      <c r="R4" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="S4" s="4" t="n">
-        <v>0.6672</v>
-      </c>
-      <c r="T4" t="n">
-        <v>0.0606</v>
-      </c>
-      <c r="U4" s="4" t="n">
-        <v>0.8336</v>
-      </c>
-      <c r="V4" t="n">
-        <v>0.0321</v>
-      </c>
-      <c r="W4" t="n">
-        <v>46.4</v>
-      </c>
-      <c r="X4" s="4" t="n">
-        <v>0.836</v>
-      </c>
-      <c r="Y4" s="4" t="n">
-        <v>0.9167999999999999</v>
-      </c>
-      <c r="Z4" s="4" t="n">
-        <v>0.9223</v>
-      </c>
-      <c r="AA4" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_epistatic_LINEAR/GB1_epistatic_cv_loss_curves.png</t>
-        </is>
-      </c>
-      <c r="AB4" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_epistatic_LINEAR/GB1_epistatic_predicted_vs_actual_test.png</t>
-        </is>
-      </c>
-      <c r="AC4" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_epistatic_LINEAR/GB1_epistatic_integrated_gradients_heatmap.png</t>
-        </is>
-      </c>
-      <c r="AD4" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_epistatic_LINEAR/GB1_epistatic_integrated_gradients_analysis.png</t>
-        </is>
-      </c>
-      <c r="AE4" t="inlineStr">
-        <is>
-          <t>Will: higher LR and DrpOut</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="n">
-        <v>4</v>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>2026-04-17 13:58</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>GB1_epistatic</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>python scripts/run_integrated_gradients.py configs/synthetic/GB1_epistatic_config.yaml</t>
-        </is>
-      </c>
-      <c r="F5" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_epistatic_LINEAR/GB1_epistatic_config_snapshot_20260417_135449.yaml</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_epistatic_LINEAR</t>
-        </is>
-      </c>
-      <c r="H5" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_epistatic_LINEAR/GB1_epistatic_run_log_20260417_135240.txt</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>esm_attention</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>128-64-32-16</t>
-        </is>
-      </c>
-      <c r="K5" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="L5" t="n">
-        <v>0.0005</v>
-      </c>
-      <c r="M5" t="n">
-        <v>64</v>
-      </c>
-      <c r="N5" t="n">
-        <v>50</v>
-      </c>
-      <c r="O5" t="n">
-        <v>10</v>
-      </c>
-      <c r="P5" t="n">
-        <v>15</v>
-      </c>
-      <c r="Q5" t="inlineStr">
-        <is>
-          <t>huber</t>
-        </is>
-      </c>
-      <c r="R5" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="S5" s="4" t="n">
-        <v>0.7254</v>
-      </c>
-      <c r="T5" t="n">
-        <v>0.016</v>
-      </c>
-      <c r="U5" s="4" t="n">
-        <v>0.8688</v>
-      </c>
-      <c r="V5" t="n">
-        <v>0.0057</v>
-      </c>
-      <c r="W5" t="n">
-        <v>44.6</v>
-      </c>
-      <c r="X5" s="4" t="n">
-        <v>0.8325</v>
-      </c>
-      <c r="Y5" s="4" t="n">
-        <v>0.9127</v>
-      </c>
-      <c r="Z5" s="4" t="n">
-        <v>0.8988</v>
-      </c>
-      <c r="AA5" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_epistatic_LINEAR/GB1_epistatic_cv_loss_curves.png</t>
-        </is>
-      </c>
-      <c r="AB5" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_epistatic_LINEAR/GB1_epistatic_predicted_vs_actual_test.png</t>
-        </is>
-      </c>
-      <c r="AC5" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_epistatic_LINEAR/GB1_epistatic_integrated_gradients_heatmap.png</t>
-        </is>
-      </c>
-      <c r="AD5" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_epistatic_LINEAR/GB1_epistatic_integrated_gradients_analysis.png</t>
-        </is>
-      </c>
-      <c r="AE5" t="inlineStr">
-        <is>
-          <t>Will: lower LR and DrpOut</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="n">
-        <v>5</v>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>2026-04-17 14:04</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>GB1_epistatic</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>python scripts/run_integrated_gradients.py configs/synthetic/GB1_epistatic_config.yaml</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_epistatic_LINEAR/GB1_epistatic_config_snapshot_20260417_135904.yaml</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_epistatic_LINEAR</t>
-        </is>
-      </c>
-      <c r="H6" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_epistatic_LINEAR/GB1_epistatic_run_log_20260417_135904.txt</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>esm_attention</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>128-64-32-16</t>
-        </is>
-      </c>
-      <c r="K6" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="L6" t="n">
-        <v>0.0005</v>
-      </c>
-      <c r="M6" t="n">
-        <v>64</v>
-      </c>
-      <c r="N6" t="n">
-        <v>50</v>
-      </c>
-      <c r="O6" t="n">
-        <v>10</v>
-      </c>
-      <c r="P6" t="n">
-        <v>15</v>
-      </c>
-      <c r="Q6" t="inlineStr">
-        <is>
-          <t>huber</t>
-        </is>
-      </c>
-      <c r="R6" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="S6" s="4" t="n">
-        <v>0.7047</v>
-      </c>
-      <c r="T6" t="n">
-        <v>0.0239</v>
-      </c>
-      <c r="U6" s="4" t="n">
-        <v>0.8567</v>
-      </c>
-      <c r="V6" t="n">
-        <v>0.0158</v>
-      </c>
-      <c r="W6" t="n">
-        <v>47</v>
-      </c>
-      <c r="X6" s="4" t="n">
-        <v>0.8169</v>
-      </c>
-      <c r="Y6" s="4" t="n">
-        <v>0.9041</v>
-      </c>
-      <c r="Z6" s="4" t="n">
-        <v>0.8878</v>
-      </c>
-      <c r="AA6" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_epistatic_LINEAR/GB1_epistatic_cv_loss_curves.png</t>
-        </is>
-      </c>
-      <c r="AB6" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_epistatic_LINEAR/GB1_epistatic_predicted_vs_actual_test.png</t>
-        </is>
-      </c>
-      <c r="AC6" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_epistatic_LINEAR/GB1_epistatic_integrated_gradients_heatmap.png</t>
-        </is>
-      </c>
-      <c r="AD6" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_epistatic_LINEAR/GB1_epistatic_integrated_gradients_analysis.png</t>
-        </is>
-      </c>
-      <c r="AE6" t="inlineStr">
-        <is>
-          <t>Will: half initial hidden dims</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H2" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA2" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB2" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC2" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD2" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F3" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H3" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA3" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB3" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC3" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD3" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F4" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H4" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA4" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB4" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC4" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD4" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F5" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H5" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA5" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB5" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC5" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD5" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F6" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA6" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB6" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC6" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD6" r:id="rId30"/>
-  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4671,7 +2953,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE6"/>
+  <dimension ref="A1:AE1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -4864,649 +3146,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>2026-04-17 13:17</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>GB1_nonlinear</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>python scripts/run_integrated_gradients.py configs/synthetic/GB1_nonlinear_config.yaml</t>
-        </is>
-      </c>
-      <c r="F2" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_nonlinear_LINEAR/GB1_nonlinear_config_snapshot_20260416_123745.yaml</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_nonlinear_LINEAR</t>
-        </is>
-      </c>
-      <c r="H2" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_nonlinear_LINEAR/GB1_nonlinear_run_log_20260416_123745.txt</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>esm_attention</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>256-128-64-32</t>
-        </is>
-      </c>
-      <c r="K2" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="L2" t="n">
-        <v>0.001</v>
-      </c>
-      <c r="M2" t="n">
-        <v>64</v>
-      </c>
-      <c r="N2" t="n">
-        <v>50</v>
-      </c>
-      <c r="O2" t="n">
-        <v>10</v>
-      </c>
-      <c r="P2" t="n">
-        <v>15</v>
-      </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>huber</t>
-        </is>
-      </c>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="S2" s="4" t="n">
-        <v>0.7554999999999999</v>
-      </c>
-      <c r="T2" t="n">
-        <v>0.0163</v>
-      </c>
-      <c r="U2" s="4" t="n">
-        <v>0.8843</v>
-      </c>
-      <c r="V2" t="n">
-        <v>0.009299999999999999</v>
-      </c>
-      <c r="W2" t="n">
-        <v>45.4</v>
-      </c>
-      <c r="X2" s="4" t="n">
-        <v>0.8066</v>
-      </c>
-      <c r="Y2" s="4" t="n">
-        <v>0.8996</v>
-      </c>
-      <c r="Z2" s="4" t="n">
-        <v>0.9005</v>
-      </c>
-      <c r="AA2" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_nonlinear_LINEAR/GB1_nonlinear_cv_loss_curves.png</t>
-        </is>
-      </c>
-      <c r="AB2" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_nonlinear_LINEAR/GB1_nonlinear_predicted_vs_actual_test.png</t>
-        </is>
-      </c>
-      <c r="AC2" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_nonlinear_LINEAR/GB1_nonlinear_integrated_gradients_heatmap.png</t>
-        </is>
-      </c>
-      <c r="AD2" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_nonlinear_LINEAR/GB1_nonlinear_integrated_gradients_analysis.png</t>
-        </is>
-      </c>
-      <c r="AE2" t="inlineStr">
-        <is>
-          <t>Will: initial run</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>2026-04-17 13:36</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>GB1_nonlinear</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>python scripts/run_integrated_gradients.py configs/synthetic/GB1_nonlinear_config.yaml</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_nonlinear_LINEAR/GB1_nonlinear_config_snapshot_20260417_133148.yaml</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_nonlinear_LINEAR</t>
-        </is>
-      </c>
-      <c r="H3" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_nonlinear_LINEAR/GB1_nonlinear_run_log_20260417_133148.txt</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>esm_attention</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>512-256-128-64</t>
-        </is>
-      </c>
-      <c r="K3" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="L3" t="n">
-        <v>0.001</v>
-      </c>
-      <c r="M3" t="n">
-        <v>64</v>
-      </c>
-      <c r="N3" t="n">
-        <v>50</v>
-      </c>
-      <c r="O3" t="n">
-        <v>10</v>
-      </c>
-      <c r="P3" t="n">
-        <v>15</v>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>huber</t>
-        </is>
-      </c>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="S3" s="4" t="n">
-        <v>0.7586000000000001</v>
-      </c>
-      <c r="T3" t="n">
-        <v>0.0268</v>
-      </c>
-      <c r="U3" s="4" t="n">
-        <v>0.8848</v>
-      </c>
-      <c r="V3" t="n">
-        <v>0.0197</v>
-      </c>
-      <c r="W3" t="n">
-        <v>45.4</v>
-      </c>
-      <c r="X3" s="4" t="n">
-        <v>0.7991</v>
-      </c>
-      <c r="Y3" s="4" t="n">
-        <v>0.8942</v>
-      </c>
-      <c r="Z3" s="4" t="n">
-        <v>0.8804</v>
-      </c>
-      <c r="AA3" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_nonlinear_LINEAR/GB1_nonlinear_cv_loss_curves.png</t>
-        </is>
-      </c>
-      <c r="AB3" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_nonlinear_LINEAR/GB1_nonlinear_predicted_vs_actual_test.png</t>
-        </is>
-      </c>
-      <c r="AC3" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_nonlinear_LINEAR/GB1_nonlinear_integrated_gradients_heatmap.png</t>
-        </is>
-      </c>
-      <c r="AD3" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_nonlinear_LINEAR/GB1_nonlinear_integrated_gradients_analysis.png</t>
-        </is>
-      </c>
-      <c r="AE3" t="inlineStr">
-        <is>
-          <t>Will: Double hidden dims</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>2026-04-17 13:51</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>GB1_nonlinear</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>python scripts/run_integrated_gradients.py configs/synthetic/GB1_nonlinear_config.yaml</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_nonlinear_LINEAR/GB1_nonlinear_config_snapshot_20260417_134434.yaml</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_nonlinear_LINEAR</t>
-        </is>
-      </c>
-      <c r="H4" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_nonlinear_LINEAR/GB1_nonlinear_run_log_20260417_134434.txt</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>esm_attention</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>512-256-128-64</t>
-        </is>
-      </c>
-      <c r="K4" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="L4" t="n">
-        <v>0.005</v>
-      </c>
-      <c r="M4" t="n">
-        <v>64</v>
-      </c>
-      <c r="N4" t="n">
-        <v>50</v>
-      </c>
-      <c r="O4" t="n">
-        <v>10</v>
-      </c>
-      <c r="P4" t="n">
-        <v>15</v>
-      </c>
-      <c r="Q4" t="inlineStr">
-        <is>
-          <t>huber</t>
-        </is>
-      </c>
-      <c r="R4" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="S4" s="4" t="n">
-        <v>0.5883</v>
-      </c>
-      <c r="T4" t="n">
-        <v>0.0663</v>
-      </c>
-      <c r="U4" s="4" t="n">
-        <v>0.7996</v>
-      </c>
-      <c r="V4" t="n">
-        <v>0.0408</v>
-      </c>
-      <c r="W4" t="n">
-        <v>41.4</v>
-      </c>
-      <c r="X4" s="4" t="n">
-        <v>0.7616000000000001</v>
-      </c>
-      <c r="Y4" s="4" t="n">
-        <v>0.8749</v>
-      </c>
-      <c r="Z4" s="4" t="n">
-        <v>0.8973</v>
-      </c>
-      <c r="AA4" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_nonlinear_LINEAR/GB1_nonlinear_cv_loss_curves.png</t>
-        </is>
-      </c>
-      <c r="AB4" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_nonlinear_LINEAR/GB1_nonlinear_predicted_vs_actual_test.png</t>
-        </is>
-      </c>
-      <c r="AC4" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_nonlinear_LINEAR/GB1_nonlinear_integrated_gradients_heatmap.png</t>
-        </is>
-      </c>
-      <c r="AD4" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_nonlinear_LINEAR/GB1_nonlinear_integrated_gradients_analysis.png</t>
-        </is>
-      </c>
-      <c r="AE4" t="inlineStr">
-        <is>
-          <t>Will: higher LR and DrpOut</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="n">
-        <v>4</v>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>2026-04-17 13:58</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>GB1_nonlinear</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>python scripts/run_integrated_gradients.py configs/synthetic/GB1_nonlinear_config.yaml</t>
-        </is>
-      </c>
-      <c r="F5" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_nonlinear_LINEAR/GB1_nonlinear_config_snapshot_20260417_135447.yaml</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_nonlinear_LINEAR</t>
-        </is>
-      </c>
-      <c r="H5" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_nonlinear_LINEAR/GB1_nonlinear_run_log_20260417_135241.txt</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>esm_attention</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>128-64-32-16</t>
-        </is>
-      </c>
-      <c r="K5" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="L5" t="n">
-        <v>0.0005</v>
-      </c>
-      <c r="M5" t="n">
-        <v>64</v>
-      </c>
-      <c r="N5" t="n">
-        <v>50</v>
-      </c>
-      <c r="O5" t="n">
-        <v>10</v>
-      </c>
-      <c r="P5" t="n">
-        <v>15</v>
-      </c>
-      <c r="Q5" t="inlineStr">
-        <is>
-          <t>huber</t>
-        </is>
-      </c>
-      <c r="R5" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="S5" s="4" t="n">
-        <v>0.7433</v>
-      </c>
-      <c r="T5" t="n">
-        <v>0.0212</v>
-      </c>
-      <c r="U5" s="4" t="n">
-        <v>0.8748</v>
-      </c>
-      <c r="V5" t="n">
-        <v>0.0127</v>
-      </c>
-      <c r="W5" t="n">
-        <v>47.6</v>
-      </c>
-      <c r="X5" s="4" t="n">
-        <v>0.8115</v>
-      </c>
-      <c r="Y5" s="4" t="n">
-        <v>0.9012</v>
-      </c>
-      <c r="Z5" s="4" t="n">
-        <v>0.8848</v>
-      </c>
-      <c r="AA5" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_nonlinear_LINEAR/GB1_nonlinear_cv_loss_curves.png</t>
-        </is>
-      </c>
-      <c r="AB5" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_nonlinear_LINEAR/GB1_nonlinear_predicted_vs_actual_test.png</t>
-        </is>
-      </c>
-      <c r="AC5" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_nonlinear_LINEAR/GB1_nonlinear_integrated_gradients_heatmap.png</t>
-        </is>
-      </c>
-      <c r="AD5" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_nonlinear_LINEAR/GB1_nonlinear_integrated_gradients_analysis.png</t>
-        </is>
-      </c>
-      <c r="AE5" t="inlineStr">
-        <is>
-          <t>Will: lower LR and DrpOut</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="n">
-        <v>5</v>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>2026-04-17 14:04</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>GB1_nonlinear</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>python scripts/run_integrated_gradients.py configs/synthetic/GB1_nonlinear_config.yaml</t>
-        </is>
-      </c>
-      <c r="F6" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_nonlinear_LINEAR/GB1_nonlinear_config_snapshot_20260417_135908.yaml</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_nonlinear_LINEAR</t>
-        </is>
-      </c>
-      <c r="H6" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_nonlinear_LINEAR/GB1_nonlinear_run_log_20260417_135908.txt</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>esm_attention</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>128-64-32-16</t>
-        </is>
-      </c>
-      <c r="K6" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="L6" t="n">
-        <v>0.0005</v>
-      </c>
-      <c r="M6" t="n">
-        <v>64</v>
-      </c>
-      <c r="N6" t="n">
-        <v>50</v>
-      </c>
-      <c r="O6" t="n">
-        <v>10</v>
-      </c>
-      <c r="P6" t="n">
-        <v>15</v>
-      </c>
-      <c r="Q6" t="inlineStr">
-        <is>
-          <t>huber</t>
-        </is>
-      </c>
-      <c r="R6" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="S6" s="4" t="n">
-        <v>0.6952</v>
-      </c>
-      <c r="T6" t="n">
-        <v>0.0324</v>
-      </c>
-      <c r="U6" s="4" t="n">
-        <v>0.847</v>
-      </c>
-      <c r="V6" t="n">
-        <v>0.0126</v>
-      </c>
-      <c r="W6" t="n">
-        <v>47.8</v>
-      </c>
-      <c r="X6" s="4" t="n">
-        <v>0.7498</v>
-      </c>
-      <c r="Y6" s="4" t="n">
-        <v>0.8693</v>
-      </c>
-      <c r="Z6" s="4" t="n">
-        <v>0.8617</v>
-      </c>
-      <c r="AA6" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_nonlinear_LINEAR/GB1_nonlinear_cv_loss_curves.png</t>
-        </is>
-      </c>
-      <c r="AB6" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_nonlinear_LINEAR/GB1_nonlinear_predicted_vs_actual_test.png</t>
-        </is>
-      </c>
-      <c r="AC6" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_nonlinear_LINEAR/GB1_nonlinear_integrated_gradients_heatmap.png</t>
-        </is>
-      </c>
-      <c r="AD6" s="3" t="inlineStr">
-        <is>
-          <t>results/synthetic/GB1_nonlinear_LINEAR/GB1_nonlinear_integrated_gradients_analysis.png</t>
-        </is>
-      </c>
-      <c r="AE6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Will: half initial hidden dims </t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H2" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA2" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB2" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC2" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD2" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F3" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H3" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA3" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB3" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC3" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD3" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F4" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H4" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA4" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB4" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC4" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD4" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F5" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H5" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA5" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB5" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC5" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD5" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F6" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA6" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB6" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC6" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD6" r:id="rId30"/>
-  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>